<commit_message>
update: tribe avatar regeneration, campaign, docs, tests, and site
</commit_message>
<xml_diff>
--- a/outputs/2fa3c415-ff27-4ff2-ae6f-40f45baa0dd4/identity_art_orders_nations_200_draft.xlsx
+++ b/outputs/2fa3c415-ff27-4ff2-ae6f-40f45baa0dd4/identity_art_orders_nations_200_draft.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selección 200" sheetId="1" r:id="R30d0601e3cb0457d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selection 200" sheetId="1" r:id="R30d0601e3cb0457d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -469,7 +469,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="28" t="str">
-        <x:v>200 identidades históricas para bots Nation</x:v>
+        <x:v>200 historical identities for Nation bots</x:v>
       </x:c>
       <x:c r="B1" s="29"/>
       <x:c r="C1" s="29"/>
@@ -480,7 +480,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="30" t="str">
-        <x:v>Selección nueva para avatares estáticos de bots; borrador para revisión. 100 mujeres y 100 hombres.</x:v>
+        <x:v>New selection for static bot avatars; draft for review. 100 women and 100 men.</x:v>
       </x:c>
       <x:c r="B2" s="29"/>
       <x:c r="C2" s="29"/>
@@ -492,30 +492,30 @@
     <x:row r="4">
       <x:c r="A4" s="29"/>
       <x:c r="B4" s="15" t="str">
-        <x:v>Composición</x:v>
+        <x:v>Composition</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>Personas</x:v>
+        <x:v>People</x:v>
       </x:c>
       <x:c r="D4" s="29"/>
       <x:c r="E4" s="15" t="str">
-        <x:v>Cobertura regional</x:v>
+        <x:v>Regional coverage</x:v>
       </x:c>
       <x:c r="F4" s="16" t="str">
-        <x:v>Personas</x:v>
+        <x:v>People</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="29"/>
       <x:c r="B5" s="31" t="str">
-        <x:v>Mujeres</x:v>
+        <x:v>Women</x:v>
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="D5" s="29"/>
       <x:c r="E5" s="31" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="F5" s="32" t="n">
         <x:v>40</x:v>
@@ -524,14 +524,14 @@
     <x:row r="6">
       <x:c r="A6" s="29"/>
       <x:c r="B6" s="33" t="str">
-        <x:v>Hombres</x:v>
+        <x:v>Men</x:v>
       </x:c>
       <x:c r="C6" s="34" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="D6" s="29"/>
       <x:c r="E6" s="31" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="F6" s="32" t="n">
         <x:v>48</x:v>
@@ -555,7 +555,7 @@
       <x:c r="C8" s="29"/>
       <x:c r="D8" s="29"/>
       <x:c r="E8" s="31" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="F8" s="32" t="n">
         <x:v>40</x:v>
@@ -567,7 +567,7 @@
       <x:c r="C9" s="29"/>
       <x:c r="D9" s="29"/>
       <x:c r="E9" s="33" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="F9" s="34" t="n">
         <x:v>16</x:v>
@@ -575,7 +575,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="35" t="str">
-        <x:v>La proporción 50/50 es una decisión de representación del roster del juego, no una afirmación sobre la proporción histórica de líderes.</x:v>
+        <x:v>The 50/50 split is a representation decision for the game roster, not a claim about the historical proportion of leaders.</x:v>
       </x:c>
       <x:c r="B10" s="29"/>
       <x:c r="C10" s="29"/>
@@ -585,7 +585,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="35" t="str">
-        <x:v>Cada registro enlaza a una referencia individual; los nombres y el orden son una propuesta, no una aprobación final.</x:v>
+        <x:v>Each record links to an individual reference; names and order are a proposal, not final approval.</x:v>
       </x:c>
       <x:c r="B11" s="29"/>
       <x:c r="C11" s="29"/>
@@ -595,25 +595,25 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="21" t="str">
-        <x:v>N.º</x:v>
+        <x:v>No.</x:v>
       </x:c>
       <x:c r="B13" s="21" t="str">
-        <x:v>Identidad</x:v>
+        <x:v>Identity</x:v>
       </x:c>
       <x:c r="C13" s="21" t="str">
-        <x:v>Género</x:v>
+        <x:v>Gender</x:v>
       </x:c>
       <x:c r="D13" s="21" t="str">
-        <x:v>Región mundial</x:v>
+        <x:v>World region</x:v>
       </x:c>
       <x:c r="E13" s="21" t="str">
-        <x:v>Entidad / pueblo asociado</x:v>
+        <x:v>Associated entity / people</x:v>
       </x:c>
       <x:c r="F13" s="21" t="str">
-        <x:v>Referencia</x:v>
+        <x:v>Reference</x:v>
       </x:c>
       <x:c r="G13" s="21" t="str">
-        <x:v>Enlace</x:v>
+        <x:v>Link</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="21" customHeight="1">
@@ -624,16 +624,16 @@
         <x:v>Hatshepsut</x:v>
       </x:c>
       <x:c r="C14" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D14" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>Egipto antiguo</x:v>
+        <x:v>Ancient Egypt</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>Wikipedia (inglés): Hatshepsut</x:v>
+        <x:v>Wikipedia (English): Hatshepsut</x:v>
       </x:c>
       <x:c r="G14" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Hatshepsut</x:v>
@@ -647,16 +647,16 @@
         <x:v>Mansa Musa</x:v>
       </x:c>
       <x:c r="C15" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D15" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Imperio de Mali</x:v>
+        <x:v>Mali Empire</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>Wikipedia (inglés): Mansa Musa</x:v>
+        <x:v>Wikipedia (English): Mansa Musa</x:v>
       </x:c>
       <x:c r="G15" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Mansa_Musa</x:v>
@@ -670,16 +670,16 @@
         <x:v>Amanirenas</x:v>
       </x:c>
       <x:c r="C16" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D16" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>Reino de Kush</x:v>
+        <x:v>Kingdom of Kush</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>Wikipedia (inglés): Amanirenas</x:v>
+        <x:v>Wikipedia (English): Amanirenas</x:v>
       </x:c>
       <x:c r="G16" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Amanirenas</x:v>
@@ -693,16 +693,16 @@
         <x:v>Sundiata Keita</x:v>
       </x:c>
       <x:c r="C17" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D17" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>Imperio de Mali</x:v>
+        <x:v>Mali Empire</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sundiata Keita</x:v>
+        <x:v>Wikipedia (English): Sundiata Keita</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sundiata_Keita</x:v>
@@ -716,16 +716,16 @@
         <x:v>Amanitore</x:v>
       </x:c>
       <x:c r="C18" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D18" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>Reino de Kush</x:v>
+        <x:v>Kingdom of Kush</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>Wikipedia (inglés): Amanitore</x:v>
+        <x:v>Wikipedia (English): Amanitore</x:v>
       </x:c>
       <x:c r="G18" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Amanitore</x:v>
@@ -736,19 +736,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Sunni Ali</x:v>
+        <x:v>Sonni Ali</x:v>
       </x:c>
       <x:c r="C19" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D19" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>Imperio songhai</x:v>
+        <x:v>Songhai Empire</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sonni Ali</x:v>
+        <x:v>Wikipedia (English): Sonni Ali</x:v>
       </x:c>
       <x:c r="G19" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sonni_Ali</x:v>
@@ -762,16 +762,16 @@
         <x:v>Amanishakheto</x:v>
       </x:c>
       <x:c r="C20" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D20" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>Reino de Kush</x:v>
+        <x:v>Kingdom of Kush</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>Wikipedia (inglés): Amanishakheto</x:v>
+        <x:v>Wikipedia (English): Amanishakheto</x:v>
       </x:c>
       <x:c r="G20" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Amanishakheto</x:v>
@@ -785,16 +785,16 @@
         <x:v>Askia Muhammad I</x:v>
       </x:c>
       <x:c r="C21" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D21" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>Imperio songhai</x:v>
+        <x:v>Songhai Empire</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>Wikipedia (inglés): Askia Muhammad I</x:v>
+        <x:v>Wikipedia (English): Askia Muhammad I</x:v>
       </x:c>
       <x:c r="G21" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Askia_Muhammad_I</x:v>
@@ -805,19 +805,19 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>Cleopatra VII</x:v>
+        <x:v>Cleopatra</x:v>
       </x:c>
       <x:c r="C22" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D22" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>Egipto ptolemaico</x:v>
+        <x:v>Ptolemaic Egypt</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>Wikipedia (inglés): Cleopatra</x:v>
+        <x:v>Wikipedia (English): Cleopatra</x:v>
       </x:c>
       <x:c r="G22" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Cleopatra</x:v>
@@ -828,19 +828,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Shaka Zulu</x:v>
+        <x:v>Shaka</x:v>
       </x:c>
       <x:c r="C23" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D23" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>Reino zulú</x:v>
+        <x:v>Zulu Kingdom</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>Wikipedia (inglés): Shaka</x:v>
+        <x:v>Wikipedia (English): Shaka</x:v>
       </x:c>
       <x:c r="G23" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Shaka</x:v>
@@ -854,16 +854,16 @@
         <x:v>Cleopatra Selene II</x:v>
       </x:c>
       <x:c r="C24" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D24" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>Mauritania antigua</x:v>
+        <x:v>Ancient Mauretania</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>Wikipedia (inglés): Cleopatra Selene II</x:v>
+        <x:v>Wikipedia (English): Cleopatra Selene II</x:v>
       </x:c>
       <x:c r="G24" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Cleopatra_Selene_II</x:v>
@@ -877,16 +877,16 @@
         <x:v>Menelik II</x:v>
       </x:c>
       <x:c r="C25" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D25" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>Etiopía</x:v>
+        <x:v>Ethiopia</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>Wikipedia (inglés): Menelik II</x:v>
+        <x:v>Wikipedia (English): Menelik II</x:v>
       </x:c>
       <x:c r="G25" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Menelik_II</x:v>
@@ -897,19 +897,19 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Nzinga Mbande</x:v>
+        <x:v>Nzinga of Ndongo and Matamba</x:v>
       </x:c>
       <x:c r="C26" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D26" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>Ndongo y Matamba</x:v>
+        <x:v>Ndongo and Matamba</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>Wikipedia (inglés): Nzinga of Ndongo and Matamba</x:v>
+        <x:v>Wikipedia (English): Nzinga of Ndongo and Matamba</x:v>
       </x:c>
       <x:c r="G26" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Nzinga_of_Ndongo_and_Matamba</x:v>
@@ -923,16 +923,16 @@
         <x:v>Haile Selassie</x:v>
       </x:c>
       <x:c r="C27" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D27" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>Etiopía</x:v>
+        <x:v>Ethiopia</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>Wikipedia (inglés): Haile Selassie</x:v>
+        <x:v>Wikipedia (English): Haile Selassie</x:v>
       </x:c>
       <x:c r="G27" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Haile_Selassie</x:v>
@@ -943,19 +943,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Amina de Zazzau</x:v>
+        <x:v>Amina of Zazzau</x:v>
       </x:c>
       <x:c r="C28" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D28" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>Zazzau (Nigeria actual)</x:v>
+        <x:v>Zazzau (modern Nigeria)</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>Wikipedia (inglés): Amina of Zazzau</x:v>
+        <x:v>Wikipedia (English): Amina of Zazzau</x:v>
       </x:c>
       <x:c r="G28" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Amina_of_Zazzau</x:v>
@@ -969,16 +969,16 @@
         <x:v>Samori Ture</x:v>
       </x:c>
       <x:c r="C29" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D29" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>Imperio Wassoulou</x:v>
+        <x:v>Wassoulou Empire</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>Wikipedia (inglés): Samori Ture</x:v>
+        <x:v>Wikipedia (English): Samori Ture</x:v>
       </x:c>
       <x:c r="G29" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Samori_Ture</x:v>
@@ -989,19 +989,19 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Reina Idia</x:v>
+        <x:v>Idia</x:v>
       </x:c>
       <x:c r="C30" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D30" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>Reino de Benín</x:v>
+        <x:v>Kingdom of Benin</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>Wikipedia (inglés): Idia</x:v>
+        <x:v>Wikipedia (English): Idia</x:v>
       </x:c>
       <x:c r="G30" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Idia</x:v>
@@ -1012,19 +1012,19 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Osei Tutu</x:v>
+        <x:v>Osei Kofi Tutu I</x:v>
       </x:c>
       <x:c r="C31" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D31" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>Imperio Ashanti</x:v>
+        <x:v>Ashanti Empire</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>Wikipedia (inglés): Osei Kofi Tutu I</x:v>
+        <x:v>Wikipedia (English): Osei Kofi Tutu I</x:v>
       </x:c>
       <x:c r="G31" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Osei_Kofi_Tutu_I</x:v>
@@ -1038,16 +1038,16 @@
         <x:v>Yaa Asantewaa</x:v>
       </x:c>
       <x:c r="C32" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D32" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>Imperio Ashanti</x:v>
+        <x:v>Ashanti Empire</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>Wikipedia (inglés): Yaa Asantewaa</x:v>
+        <x:v>Wikipedia (English): Yaa Asantewaa</x:v>
       </x:c>
       <x:c r="G32" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Yaa_Asantewaa</x:v>
@@ -1061,16 +1061,16 @@
         <x:v>Tewodros II</x:v>
       </x:c>
       <x:c r="C33" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D33" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>Etiopía</x:v>
+        <x:v>Ethiopia</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>Wikipedia (inglés): Tewodros II</x:v>
+        <x:v>Wikipedia (English): Tewodros II</x:v>
       </x:c>
       <x:c r="G33" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tewodros_II</x:v>
@@ -1084,16 +1084,16 @@
         <x:v>Ranavalona I</x:v>
       </x:c>
       <x:c r="C34" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D34" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>Reino de Madagascar</x:v>
+        <x:v>Kingdom of Madagascar</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ranavalona I</x:v>
+        <x:v>Wikipedia (English): Ranavalona I</x:v>
       </x:c>
       <x:c r="G34" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ranavalona_I</x:v>
@@ -1107,16 +1107,16 @@
         <x:v>Ahmad al-Mansur</x:v>
       </x:c>
       <x:c r="C35" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D35" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>Marruecos / dinastía saadí</x:v>
+        <x:v>Morocco / Saadi dynasty</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ahmad al-Mansur</x:v>
+        <x:v>Wikipedia (English): Ahmad al-Mansur</x:v>
       </x:c>
       <x:c r="G35" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ahmad_al-Mansur</x:v>
@@ -1130,16 +1130,16 @@
         <x:v>Ranavalona II</x:v>
       </x:c>
       <x:c r="C36" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D36" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>Reino de Madagascar</x:v>
+        <x:v>Kingdom of Madagascar</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ranavalona II</x:v>
+        <x:v>Wikipedia (English): Ranavalona II</x:v>
       </x:c>
       <x:c r="G36" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ranavalona_II</x:v>
@@ -1153,16 +1153,16 @@
         <x:v>Idris Alooma</x:v>
       </x:c>
       <x:c r="C37" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D37" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>Imperio Kanem-Bornu</x:v>
+        <x:v>Kanem-Bornu Empire</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>Wikipedia (inglés): Idris Alooma</x:v>
+        <x:v>Wikipedia (English): Idris Alooma</x:v>
       </x:c>
       <x:c r="G37" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Idris_Alooma</x:v>
@@ -1173,19 +1173,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>Dihya</x:v>
+        <x:v>Kahina</x:v>
       </x:c>
       <x:c r="C38" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D38" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>Aures y pueblos amazigh</x:v>
+        <x:v>Aurès and Amazigh peoples</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>Wikipedia (inglés): Kahina</x:v>
+        <x:v>Wikipedia (English): Kahina</x:v>
       </x:c>
       <x:c r="G38" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Kahina</x:v>
@@ -1196,19 +1196,19 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Omar Mukhtar</x:v>
+        <x:v>Omar al-Mukhtar</x:v>
       </x:c>
       <x:c r="C39" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D39" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>Libia</x:v>
+        <x:v>Libya</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>Wikipedia (inglés): Omar al-Mukhtar</x:v>
+        <x:v>Wikipedia (English): Omar al-Mukhtar</x:v>
       </x:c>
       <x:c r="G39" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Omar_al-Mukhtar</x:v>
@@ -1222,16 +1222,16 @@
         <x:v>Nehanda Charwe Nyakasikana</x:v>
       </x:c>
       <x:c r="C40" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D40" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>Zimbabue / Shona</x:v>
+        <x:v>Zimbabwe / Shona</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>Wikipedia (inglés): Nehanda Charwe Nyakasikana</x:v>
+        <x:v>Wikipedia (English): Nehanda Charwe Nyakasikana</x:v>
       </x:c>
       <x:c r="G40" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Nehanda_Charwe_Nyakasikana</x:v>
@@ -1242,19 +1242,19 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Mutesa I de Buganda</x:v>
+        <x:v>Muteesa I of Buganda</x:v>
       </x:c>
       <x:c r="C41" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D41" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>Reino de Buganda</x:v>
+        <x:v>Kingdom of Buganda</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>Wikipedia (inglés): Muteesa I of Buganda</x:v>
+        <x:v>Wikipedia (English): Muteesa I of Buganda</x:v>
       </x:c>
       <x:c r="G41" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Muteesa_I_of_Buganda</x:v>
@@ -1268,16 +1268,16 @@
         <x:v>Lalla Fatma N'Soumer</x:v>
       </x:c>
       <x:c r="C42" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D42" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>Cabilia (Argelia)</x:v>
+        <x:v>Kabylia (Algeria)</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>Wikipedia (inglés): Lalla Fatma N'Soumer</x:v>
+        <x:v>Wikipedia (English): Lalla Fatma N'Soumer</x:v>
       </x:c>
       <x:c r="G42" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lalla_Fatma_N%27Soumer</x:v>
@@ -1291,16 +1291,16 @@
         <x:v>Dingane</x:v>
       </x:c>
       <x:c r="C43" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D43" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>Reino zulú</x:v>
+        <x:v>Zulu Kingdom</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>Wikipedia (inglés): Dingane</x:v>
+        <x:v>Wikipedia (English): Dingane</x:v>
       </x:c>
       <x:c r="G43" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Dingane</x:v>
@@ -1311,19 +1311,19 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Sarraounia Mangou</x:v>
+        <x:v>Sarraounia</x:v>
       </x:c>
       <x:c r="C44" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D44" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>Azna / actual Níger</x:v>
+        <x:v>Azna / modern Niger</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sarraounia</x:v>
+        <x:v>Wikipedia (English): Sarraounia</x:v>
       </x:c>
       <x:c r="G44" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sarraounia</x:v>
@@ -1337,16 +1337,16 @@
         <x:v>Cetshwayo</x:v>
       </x:c>
       <x:c r="C45" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D45" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>Reino zulú</x:v>
+        <x:v>Zulu Kingdom</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>Wikipedia (inglés): Cetshwayo</x:v>
+        <x:v>Wikipedia (English): Cetshwayo</x:v>
       </x:c>
       <x:c r="G45" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Cetshwayo</x:v>
@@ -1360,16 +1360,16 @@
         <x:v>Kimpa Vita</x:v>
       </x:c>
       <x:c r="C46" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D46" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>Reino del Congo</x:v>
+        <x:v>Kingdom of Kongo</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>Wikipedia (inglés): Kimpa Vita</x:v>
+        <x:v>Wikipedia (English): Kimpa Vita</x:v>
       </x:c>
       <x:c r="G46" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Kimpa_Vita</x:v>
@@ -1383,16 +1383,16 @@
         <x:v>Taharqa</x:v>
       </x:c>
       <x:c r="C47" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D47" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>Reino de Kush</x:v>
+        <x:v>Kingdom of Kush</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>Wikipedia (inglés): Taharqa</x:v>
+        <x:v>Wikipedia (English): Taharqa</x:v>
       </x:c>
       <x:c r="G47" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Taharqa</x:v>
@@ -1406,16 +1406,16 @@
         <x:v>Labotsibeni Mdluli</x:v>
       </x:c>
       <x:c r="C48" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D48" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>Suazilandia / Esuatini</x:v>
+        <x:v>Eswatini</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>Wikipedia (inglés): Labotsibeni Mdluli</x:v>
+        <x:v>Wikipedia (English): Labotsibeni Mdluli</x:v>
       </x:c>
       <x:c r="G48" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Labotsibeni_Mdluli</x:v>
@@ -1429,16 +1429,16 @@
         <x:v>Piye</x:v>
       </x:c>
       <x:c r="C49" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D49" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>Reino de Kush</x:v>
+        <x:v>Kingdom of Kush</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>Wikipedia (inglés): Piye</x:v>
+        <x:v>Wikipedia (English): Piye</x:v>
       </x:c>
       <x:c r="G49" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Piye</x:v>
@@ -1452,16 +1452,16 @@
         <x:v>Zewditu</x:v>
       </x:c>
       <x:c r="C50" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D50" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E50" s="23" t="str">
-        <x:v>Etiopía</x:v>
+        <x:v>Ethiopia</x:v>
       </x:c>
       <x:c r="F50" s="23" t="str">
-        <x:v>Wikipedia (inglés): Zewditu</x:v>
+        <x:v>Wikipedia (English): Zewditu</x:v>
       </x:c>
       <x:c r="G50" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Zewditu</x:v>
@@ -1475,16 +1475,16 @@
         <x:v>Maqoma</x:v>
       </x:c>
       <x:c r="C51" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D51" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E51" s="23" t="str">
-        <x:v>Pueblo xhosa</x:v>
+        <x:v>Xhosa people</x:v>
       </x:c>
       <x:c r="F51" s="23" t="str">
-        <x:v>Wikipedia (inglés): Maqoma</x:v>
+        <x:v>Wikipedia (English): Maqoma</x:v>
       </x:c>
       <x:c r="G51" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Maqoma</x:v>
@@ -1498,16 +1498,16 @@
         <x:v>Taytu Betul</x:v>
       </x:c>
       <x:c r="C52" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D52" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
-        <x:v>Etiopía</x:v>
+        <x:v>Ethiopia</x:v>
       </x:c>
       <x:c r="F52" s="23" t="str">
-        <x:v>Wikipedia (inglés): Taytu Betul</x:v>
+        <x:v>Wikipedia (English): Taytu Betul</x:v>
       </x:c>
       <x:c r="G52" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Taytu_Betul</x:v>
@@ -1518,19 +1518,19 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B53" s="23" t="str">
-        <x:v>Ewuare el Grande</x:v>
+        <x:v>Ewuare</x:v>
       </x:c>
       <x:c r="C53" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D53" s="22" t="str">
-        <x:v>África</x:v>
+        <x:v>Africa</x:v>
       </x:c>
       <x:c r="E53" s="23" t="str">
-        <x:v>Reino de Benín</x:v>
+        <x:v>Kingdom of Benin</x:v>
       </x:c>
       <x:c r="F53" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ewuare</x:v>
+        <x:v>Wikipedia (English): Ewuare</x:v>
       </x:c>
       <x:c r="G53" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ewuare</x:v>
@@ -1544,16 +1544,16 @@
         <x:v>Anacaona</x:v>
       </x:c>
       <x:c r="C54" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D54" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E54" s="23" t="str">
-        <x:v>Xaragua / pueblo taíno</x:v>
+        <x:v>Xaragua / Taíno people</x:v>
       </x:c>
       <x:c r="F54" s="23" t="str">
-        <x:v>Wikipedia (inglés): Anacaona</x:v>
+        <x:v>Wikipedia (English): Anacaona</x:v>
       </x:c>
       <x:c r="G54" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Anacaona</x:v>
@@ -1567,16 +1567,16 @@
         <x:v>Moctezuma I</x:v>
       </x:c>
       <x:c r="C55" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D55" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E55" s="23" t="str">
-        <x:v>Imperio mexica</x:v>
+        <x:v>Mexica Empire</x:v>
       </x:c>
       <x:c r="F55" s="23" t="str">
-        <x:v>Wikipedia (inglés): Moctezuma I</x:v>
+        <x:v>Wikipedia (English): Moctezuma I</x:v>
       </x:c>
       <x:c r="G55" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Moctezuma_I</x:v>
@@ -1590,16 +1590,16 @@
         <x:v>Lady Six Sky</x:v>
       </x:c>
       <x:c r="C56" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D56" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E56" s="23" t="str">
-        <x:v>Naranjo / mundo maya</x:v>
+        <x:v>Naranjo</x:v>
       </x:c>
       <x:c r="F56" s="23" t="str">
-        <x:v>Wikipedia (inglés): Lady Six Sky</x:v>
+        <x:v>Wikipedia (English): Lady Six Sky</x:v>
       </x:c>
       <x:c r="G56" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lady_Six_Sky</x:v>
@@ -1613,16 +1613,16 @@
         <x:v>Moctezuma II</x:v>
       </x:c>
       <x:c r="C57" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D57" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E57" s="23" t="str">
-        <x:v>Imperio mexica</x:v>
+        <x:v>Mexica Empire</x:v>
       </x:c>
       <x:c r="F57" s="23" t="str">
-        <x:v>Wikipedia (inglés): Moctezuma II</x:v>
+        <x:v>Wikipedia (English): Moctezuma II</x:v>
       </x:c>
       <x:c r="G57" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Moctezuma_II</x:v>
@@ -1633,19 +1633,19 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B58" s="23" t="str">
-        <x:v>Lady Yohl Ik'nal</x:v>
+        <x:v>Yohl Ikʼnal</x:v>
       </x:c>
       <x:c r="C58" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D58" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E58" s="23" t="str">
-        <x:v>Palenque / mundo maya</x:v>
+        <x:v>Palenque / Maya world</x:v>
       </x:c>
       <x:c r="F58" s="23" t="str">
-        <x:v>Wikipedia (inglés): Yohl Ikʼnal</x:v>
+        <x:v>Wikipedia (English): Yohl Ikʼnal</x:v>
       </x:c>
       <x:c r="G58" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Yohl_Ik%CA%BCnal</x:v>
@@ -1659,16 +1659,16 @@
         <x:v>Atahualpa</x:v>
       </x:c>
       <x:c r="C59" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D59" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E59" s="23" t="str">
-        <x:v>Imperio inca</x:v>
+        <x:v>Inca Empire</x:v>
       </x:c>
       <x:c r="F59" s="23" t="str">
-        <x:v>Wikipedia (inglés): Atahualpa</x:v>
+        <x:v>Wikipedia (English): Atahualpa</x:v>
       </x:c>
       <x:c r="G59" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Atahualpa</x:v>
@@ -1679,19 +1679,19 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B60" s="23" t="str">
-        <x:v>Lady K'ab'al Xook</x:v>
+        <x:v>Lady Xoc</x:v>
       </x:c>
       <x:c r="C60" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D60" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E60" s="23" t="str">
-        <x:v>Yaxchilán / mundo maya</x:v>
+        <x:v>Yaxchilán / Maya world</x:v>
       </x:c>
       <x:c r="F60" s="23" t="str">
-        <x:v>Wikipedia (inglés): Lady Xoc</x:v>
+        <x:v>Wikipedia (English): Lady Xoc</x:v>
       </x:c>
       <x:c r="G60" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lady_Xoc</x:v>
@@ -1702,19 +1702,19 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B61" s="23" t="str">
-        <x:v>Pachacútec</x:v>
+        <x:v>Pachacuti</x:v>
       </x:c>
       <x:c r="C61" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D61" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E61" s="23" t="str">
-        <x:v>Imperio inca</x:v>
+        <x:v>Inca Empire</x:v>
       </x:c>
       <x:c r="F61" s="23" t="str">
-        <x:v>Wikipedia (inglés): Pachacuti</x:v>
+        <x:v>Wikipedia (English): Pachacuti</x:v>
       </x:c>
       <x:c r="G61" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Pachacuti</x:v>
@@ -1725,19 +1725,19 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B62" s="23" t="str">
-        <x:v>Lady Tz'akbu Ajaw</x:v>
+        <x:v>Tz'akbu Ajaw</x:v>
       </x:c>
       <x:c r="C62" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D62" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E62" s="23" t="str">
-        <x:v>Palenque / mundo maya</x:v>
+        <x:v>Palenque / Maya world</x:v>
       </x:c>
       <x:c r="F62" s="23" t="str">
-        <x:v>Wikipedia (inglés): Tz'akbu Ajaw</x:v>
+        <x:v>Wikipedia (English): Tz'akbu Ajaw</x:v>
       </x:c>
       <x:c r="G62" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tz%27akbu_Ajaw</x:v>
@@ -1748,19 +1748,19 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B63" s="23" t="str">
-        <x:v>Huayna Cápac</x:v>
+        <x:v>Huayna Capac</x:v>
       </x:c>
       <x:c r="C63" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D63" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E63" s="23" t="str">
-        <x:v>Imperio inca</x:v>
+        <x:v>Inca Empire</x:v>
       </x:c>
       <x:c r="F63" s="23" t="str">
-        <x:v>Wikipedia (inglés): Huayna Capac</x:v>
+        <x:v>Wikipedia (English): Huayna Capac</x:v>
       </x:c>
       <x:c r="G63" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Huayna_Capac</x:v>
@@ -1774,16 +1774,16 @@
         <x:v>Lady K'abel</x:v>
       </x:c>
       <x:c r="C64" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D64" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E64" s="23" t="str">
-        <x:v>El Perú-Waka' / mundo maya</x:v>
+        <x:v>Perú-Waka' / Maya world</x:v>
       </x:c>
       <x:c r="F64" s="23" t="str">
-        <x:v>Wikipedia (inglés): Lady K'abel</x:v>
+        <x:v>Wikipedia (English): Lady K'abel</x:v>
       </x:c>
       <x:c r="G64" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lady_K%27abel</x:v>
@@ -1794,19 +1794,19 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B65" s="23" t="str">
-        <x:v>Itzcóatl</x:v>
+        <x:v>Itzcoatl</x:v>
       </x:c>
       <x:c r="C65" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D65" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E65" s="23" t="str">
-        <x:v>Imperio mexica</x:v>
+        <x:v>Mexica Empire</x:v>
       </x:c>
       <x:c r="F65" s="23" t="str">
-        <x:v>Wikipedia (inglés): Itzcoatl</x:v>
+        <x:v>Wikipedia (English): Itzcoatl</x:v>
       </x:c>
       <x:c r="G65" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Itzcoatl</x:v>
@@ -1820,16 +1820,16 @@
         <x:v>Atotoztli</x:v>
       </x:c>
       <x:c r="C66" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D66" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E66" s="23" t="str">
-        <x:v>México-Tenochtitlan / mexica</x:v>
+        <x:v>Mexico-Tenochtitlan / Mexica</x:v>
       </x:c>
       <x:c r="F66" s="23" t="str">
-        <x:v>Wikipedia (inglés): Atotoztli</x:v>
+        <x:v>Wikipedia (English): Atotoztli</x:v>
       </x:c>
       <x:c r="G66" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Atotoztli</x:v>
@@ -1843,16 +1843,16 @@
         <x:v>Cuauhtémoc</x:v>
       </x:c>
       <x:c r="C67" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D67" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E67" s="23" t="str">
-        <x:v>Imperio mexica</x:v>
+        <x:v>Mexica Empire</x:v>
       </x:c>
       <x:c r="F67" s="23" t="str">
-        <x:v>Wikipedia (inglés): Cuauhtémoc</x:v>
+        <x:v>Wikipedia (English): Cuauhtémoc</x:v>
       </x:c>
       <x:c r="G67" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Cuauht%C3%A9moc</x:v>
@@ -1863,19 +1863,19 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B68" s="23" t="str">
-        <x:v>Tecuichpo Ixcaxochitzin</x:v>
+        <x:v>Isabel Moctezuma</x:v>
       </x:c>
       <x:c r="C68" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D68" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E68" s="23" t="str">
-        <x:v>México-Tenochtitlan / mexica</x:v>
+        <x:v>Mexico-Tenochtitlan / Mexica</x:v>
       </x:c>
       <x:c r="F68" s="23" t="str">
-        <x:v>Wikipedia (inglés): Isabel Moctezuma</x:v>
+        <x:v>Wikipedia (English): Isabel Moctezuma</x:v>
       </x:c>
       <x:c r="G68" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Isabel_Moctezuma</x:v>
@@ -1889,16 +1889,16 @@
         <x:v>Tecumseh</x:v>
       </x:c>
       <x:c r="C69" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D69" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E69" s="23" t="str">
-        <x:v>Shawnee / Confederación indígena</x:v>
+        <x:v>Shawnee / Indigenous confederacy</x:v>
       </x:c>
       <x:c r="F69" s="23" t="str">
-        <x:v>Wikipedia (inglés): Tecumseh</x:v>
+        <x:v>Wikipedia (English): Tecumseh</x:v>
       </x:c>
       <x:c r="G69" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tecumseh</x:v>
@@ -1909,19 +1909,19 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B70" s="23" t="str">
-        <x:v>Malintzin</x:v>
+        <x:v>La Malinche</x:v>
       </x:c>
       <x:c r="C70" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D70" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E70" s="23" t="str">
-        <x:v>Pueblos nahuas / México</x:v>
+        <x:v>Nahua peoples / Mexico</x:v>
       </x:c>
       <x:c r="F70" s="23" t="str">
-        <x:v>Wikipedia (inglés): La Malinche</x:v>
+        <x:v>Wikipedia (English): La Malinche</x:v>
       </x:c>
       <x:c r="G70" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/La_Malinche</x:v>
@@ -1935,16 +1935,16 @@
         <x:v>Crazy Horse</x:v>
       </x:c>
       <x:c r="C71" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D71" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E71" s="23" t="str">
         <x:v>Lakota</x:v>
       </x:c>
       <x:c r="F71" s="23" t="str">
-        <x:v>Wikipedia (inglés): Crazy Horse</x:v>
+        <x:v>Wikipedia (English): Crazy Horse</x:v>
       </x:c>
       <x:c r="G71" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Crazy_Horse</x:v>
@@ -1958,13 +1958,13 @@
         <x:v>Nanyehi (Nancy Ward)</x:v>
       </x:c>
       <x:c r="C72" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D72" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E72" s="23" t="str">
-        <x:v>Nación Cherokee</x:v>
+        <x:v>Cherokee Nation</x:v>
       </x:c>
       <x:c r="F72" s="23" t="str">
         <x:v>Colonial Williamsburg: Nancy Ward</x:v>
@@ -1981,16 +1981,16 @@
         <x:v>Red Cloud</x:v>
       </x:c>
       <x:c r="C73" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D73" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E73" s="23" t="str">
         <x:v>Lakota</x:v>
       </x:c>
       <x:c r="F73" s="23" t="str">
-        <x:v>Wikipedia (inglés): Red Cloud</x:v>
+        <x:v>Wikipedia (English): Red Cloud</x:v>
       </x:c>
       <x:c r="G73" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Red_Cloud</x:v>
@@ -2004,16 +2004,16 @@
         <x:v>Molly Brant</x:v>
       </x:c>
       <x:c r="C74" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D74" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E74" s="23" t="str">
         <x:v>Mohawk / Haudenosaunee</x:v>
       </x:c>
       <x:c r="F74" s="23" t="str">
-        <x:v>Wikipedia (inglés): Molly Brant</x:v>
+        <x:v>Wikipedia (English): Molly Brant</x:v>
       </x:c>
       <x:c r="G74" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Molly_Brant</x:v>
@@ -2027,16 +2027,16 @@
         <x:v>Sitting Bull</x:v>
       </x:c>
       <x:c r="C75" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D75" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E75" s="23" t="str">
         <x:v>Hunkpapa Lakota</x:v>
       </x:c>
       <x:c r="F75" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sitting Bull</x:v>
+        <x:v>Wikipedia (English): Sitting Bull</x:v>
       </x:c>
       <x:c r="G75" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sitting_Bull</x:v>
@@ -2050,16 +2050,16 @@
         <x:v>Lozen</x:v>
       </x:c>
       <x:c r="C76" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D76" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E76" s="23" t="str">
         <x:v>Chiricahua Apache</x:v>
       </x:c>
       <x:c r="F76" s="23" t="str">
-        <x:v>Wikipedia (inglés): Lozen</x:v>
+        <x:v>Wikipedia (English): Lozen</x:v>
       </x:c>
       <x:c r="G76" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lozen</x:v>
@@ -2073,16 +2073,16 @@
         <x:v>Geronimo</x:v>
       </x:c>
       <x:c r="C77" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D77" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E77" s="23" t="str">
         <x:v>Chiricahua Apache</x:v>
       </x:c>
       <x:c r="F77" s="23" t="str">
-        <x:v>Wikipedia (inglés): Geronimo</x:v>
+        <x:v>Wikipedia (English): Geronimo</x:v>
       </x:c>
       <x:c r="G77" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Geronimo</x:v>
@@ -2096,16 +2096,16 @@
         <x:v>Sarah Winnemucca</x:v>
       </x:c>
       <x:c r="C78" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D78" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E78" s="23" t="str">
         <x:v>Northern Paiute</x:v>
       </x:c>
       <x:c r="F78" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sarah Winnemucca</x:v>
+        <x:v>Wikipedia (English): Sarah Winnemucca</x:v>
       </x:c>
       <x:c r="G78" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sarah_Winnemucca</x:v>
@@ -2119,16 +2119,16 @@
         <x:v>Túpac Amaru II</x:v>
       </x:c>
       <x:c r="C79" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D79" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E79" s="23" t="str">
-        <x:v>Rebelión andina / Perú</x:v>
+        <x:v>Andean Rebellion / Peru</x:v>
       </x:c>
       <x:c r="F79" s="23" t="str">
-        <x:v>Wikipedia (inglés): Túpac Amaru II</x:v>
+        <x:v>Wikipedia (English): Túpac Amaru II</x:v>
       </x:c>
       <x:c r="G79" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/T%C3%BApac_Amaru_II</x:v>
@@ -2142,16 +2142,16 @@
         <x:v>Micaela Bastidas</x:v>
       </x:c>
       <x:c r="C80" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D80" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E80" s="23" t="str">
-        <x:v>Rebelión andina / Perú</x:v>
+        <x:v>Andean Rebellion / Peru</x:v>
       </x:c>
       <x:c r="F80" s="23" t="str">
-        <x:v>Wikipedia (inglés): Micaela Bastidas</x:v>
+        <x:v>Wikipedia (English): Micaela Bastidas</x:v>
       </x:c>
       <x:c r="G80" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Micaela_Bastidas</x:v>
@@ -2165,16 +2165,16 @@
         <x:v>Guaicaipuro</x:v>
       </x:c>
       <x:c r="C81" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D81" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E81" s="23" t="str">
-        <x:v>Pueblo caribe / Venezuela</x:v>
+        <x:v>Carib people / Venezuela</x:v>
       </x:c>
       <x:c r="F81" s="23" t="str">
-        <x:v>Wikipedia (inglés): Guaicaipuro</x:v>
+        <x:v>Wikipedia (English): Guaicaipuro</x:v>
       </x:c>
       <x:c r="G81" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Guaicaipuro</x:v>
@@ -2188,16 +2188,16 @@
         <x:v>Bartolina Sisa</x:v>
       </x:c>
       <x:c r="C82" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D82" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E82" s="23" t="str">
-        <x:v>Pueblo aymara / Alto Perú</x:v>
+        <x:v>Aymara people / Upper Peru</x:v>
       </x:c>
       <x:c r="F82" s="23" t="str">
-        <x:v>Wikipedia (inglés): Bartolina Sisa</x:v>
+        <x:v>Wikipedia (English): Bartolina Sisa</x:v>
       </x:c>
       <x:c r="G82" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Bartolina_Sisa</x:v>
@@ -2208,19 +2208,19 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B83" s="23" t="str">
-        <x:v>Túpac Yupanqui</x:v>
+        <x:v>Topa Inca Yupanqui</x:v>
       </x:c>
       <x:c r="C83" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D83" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E83" s="23" t="str">
-        <x:v>Imperio inca</x:v>
+        <x:v>Inca Empire</x:v>
       </x:c>
       <x:c r="F83" s="23" t="str">
-        <x:v>Wikipedia (inglés): Topa Inca Yupanqui</x:v>
+        <x:v>Wikipedia (English): Topa Inca Yupanqui</x:v>
       </x:c>
       <x:c r="G83" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Topa_Inca_Yupanqui</x:v>
@@ -2231,19 +2231,19 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B84" s="23" t="str">
-        <x:v>Juana Azurduy</x:v>
+        <x:v>Juana Azurduy de Padilla</x:v>
       </x:c>
       <x:c r="C84" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D84" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E84" s="23" t="str">
-        <x:v>Alto Perú / Bolivia</x:v>
+        <x:v>Upper Peru / Bolivia</x:v>
       </x:c>
       <x:c r="F84" s="23" t="str">
-        <x:v>Wikipedia (inglés): Juana Azurduy de Padilla</x:v>
+        <x:v>Wikipedia (English): Juana Azurduy de Padilla</x:v>
       </x:c>
       <x:c r="G84" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Juana_Azurduy_de_Padilla</x:v>
@@ -2257,16 +2257,16 @@
         <x:v>Simón Bolívar</x:v>
       </x:c>
       <x:c r="C85" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D85" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E85" s="23" t="str">
         <x:v>Gran Colombia</x:v>
       </x:c>
       <x:c r="F85" s="23" t="str">
-        <x:v>Wikipedia (inglés): Simón Bolívar</x:v>
+        <x:v>Wikipedia (English): Simón Bolívar</x:v>
       </x:c>
       <x:c r="G85" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sim%C3%B3n_Bol%C3%ADvar</x:v>
@@ -2280,16 +2280,16 @@
         <x:v>Josefa Ortiz de Domínguez</x:v>
       </x:c>
       <x:c r="C86" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D86" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E86" s="23" t="str">
-        <x:v>México</x:v>
+        <x:v>Mexico</x:v>
       </x:c>
       <x:c r="F86" s="23" t="str">
-        <x:v>Wikipedia (inglés): Josefa Ortiz de Domínguez</x:v>
+        <x:v>Wikipedia (English): Josefa Ortiz de Domínguez</x:v>
       </x:c>
       <x:c r="G86" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Josefa_Ortiz_de_Dom%C3%ADnguez</x:v>
@@ -2303,16 +2303,16 @@
         <x:v>José de San Martín</x:v>
       </x:c>
       <x:c r="C87" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D87" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E87" s="23" t="str">
-        <x:v>Argentina / Chile / Perú</x:v>
+        <x:v>Argentina / Chile / Peru</x:v>
       </x:c>
       <x:c r="F87" s="23" t="str">
-        <x:v>Wikipedia (inglés): José de San Martín</x:v>
+        <x:v>Wikipedia (English): José de San Martín</x:v>
       </x:c>
       <x:c r="G87" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Jos%C3%A9_de_San_Mart%C3%ADn</x:v>
@@ -2326,16 +2326,16 @@
         <x:v>Policarpa Salavarrieta</x:v>
       </x:c>
       <x:c r="C88" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D88" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E88" s="23" t="str">
-        <x:v>Nueva Granada / Colombia</x:v>
+        <x:v>New Granada / Colombia</x:v>
       </x:c>
       <x:c r="F88" s="23" t="str">
-        <x:v>Wikipedia (inglés): Policarpa Salavarrieta</x:v>
+        <x:v>Wikipedia (English): Policarpa Salavarrieta</x:v>
       </x:c>
       <x:c r="G88" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Policarpa_Salavarrieta</x:v>
@@ -2349,16 +2349,16 @@
         <x:v>Toussaint Louverture</x:v>
       </x:c>
       <x:c r="C89" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D89" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E89" s="23" t="str">
-        <x:v>Haití</x:v>
+        <x:v>Haiti</x:v>
       </x:c>
       <x:c r="F89" s="23" t="str">
-        <x:v>Wikipedia (inglés): Toussaint Louverture</x:v>
+        <x:v>Wikipedia (English): Toussaint Louverture</x:v>
       </x:c>
       <x:c r="G89" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Toussaint_Louverture</x:v>
@@ -2372,16 +2372,16 @@
         <x:v>Gregoria Apaza</x:v>
       </x:c>
       <x:c r="C90" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D90" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E90" s="23" t="str">
-        <x:v>Pueblo aymara / Alto Perú</x:v>
+        <x:v>Aymara people / Upper Peru</x:v>
       </x:c>
       <x:c r="F90" s="23" t="str">
-        <x:v>Wikipedia (inglés): Gregoria Apaza</x:v>
+        <x:v>Wikipedia (English): Gregoria Apaza</x:v>
       </x:c>
       <x:c r="G90" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Gregoria_Apaza</x:v>
@@ -2395,16 +2395,16 @@
         <x:v>Caupolicán</x:v>
       </x:c>
       <x:c r="C91" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D91" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E91" s="23" t="str">
-        <x:v>Pueblo mapuche</x:v>
+        <x:v>Mapuche people</x:v>
       </x:c>
       <x:c r="F91" s="23" t="str">
-        <x:v>Wikipedia (inglés): Caupolicán</x:v>
+        <x:v>Wikipedia (English): Caupolicán</x:v>
       </x:c>
       <x:c r="G91" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Caupolic%C3%A1n</x:v>
@@ -2418,16 +2418,16 @@
         <x:v>Manuela Sáenz</x:v>
       </x:c>
       <x:c r="C92" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D92" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E92" s="23" t="str">
         <x:v>Ecuador / Gran Colombia</x:v>
       </x:c>
       <x:c r="F92" s="23" t="str">
-        <x:v>Wikipedia (inglés): Manuela Sáenz</x:v>
+        <x:v>Wikipedia (English): Manuela Sáenz</x:v>
       </x:c>
       <x:c r="G92" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Manuela_S%C3%A1enz</x:v>
@@ -2441,16 +2441,16 @@
         <x:v>Lautaro</x:v>
       </x:c>
       <x:c r="C93" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D93" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E93" s="23" t="str">
-        <x:v>Pueblo mapuche</x:v>
+        <x:v>Mapuche people</x:v>
       </x:c>
       <x:c r="F93" s="23" t="str">
-        <x:v>Wikipedia (inglés): Lautaro</x:v>
+        <x:v>Wikipedia (English): Lautaro</x:v>
       </x:c>
       <x:c r="G93" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lautaro</x:v>
@@ -2464,16 +2464,16 @@
         <x:v>Isabel Perón</x:v>
       </x:c>
       <x:c r="C94" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D94" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E94" s="23" t="str">
         <x:v>Argentina</x:v>
       </x:c>
       <x:c r="F94" s="23" t="str">
-        <x:v>Wikipedia (inglés): Isabel Perón</x:v>
+        <x:v>Wikipedia (English): Isabel Perón</x:v>
       </x:c>
       <x:c r="G94" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Isabel_Per%C3%B3n</x:v>
@@ -2487,16 +2487,16 @@
         <x:v>Pontiac</x:v>
       </x:c>
       <x:c r="C95" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D95" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E95" s="23" t="str">
-        <x:v>Pueblo odawa</x:v>
+        <x:v>Odawa people</x:v>
       </x:c>
       <x:c r="F95" s="23" t="str">
-        <x:v>Wikipedia (inglés): Pontiac (Odawa leader)</x:v>
+        <x:v>Wikipedia (English): Pontiac (Odawa leader)</x:v>
       </x:c>
       <x:c r="G95" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Pontiac_(Odawa_leader)</x:v>
@@ -2510,16 +2510,16 @@
         <x:v>Violeta Chamorro</x:v>
       </x:c>
       <x:c r="C96" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D96" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E96" s="23" t="str">
         <x:v>Nicaragua</x:v>
       </x:c>
       <x:c r="F96" s="23" t="str">
-        <x:v>Wikipedia (inglés): Violeta Chamorro</x:v>
+        <x:v>Wikipedia (English): Violeta Chamorro</x:v>
       </x:c>
       <x:c r="G96" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Violeta_Chamorro</x:v>
@@ -2533,16 +2533,16 @@
         <x:v>Powhatan</x:v>
       </x:c>
       <x:c r="C97" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D97" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E97" s="23" t="str">
-        <x:v>Confederación powhatan</x:v>
+        <x:v>Powhatan Confederacy</x:v>
       </x:c>
       <x:c r="F97" s="23" t="str">
-        <x:v>Wikipedia (inglés): Powhatan</x:v>
+        <x:v>Wikipedia (English): Powhatan</x:v>
       </x:c>
       <x:c r="G97" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Powhatan</x:v>
@@ -2556,16 +2556,16 @@
         <x:v>Wilma Mankiller</x:v>
       </x:c>
       <x:c r="C98" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D98" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E98" s="23" t="str">
-        <x:v>Nación Cherokee</x:v>
+        <x:v>Cherokee Nation</x:v>
       </x:c>
       <x:c r="F98" s="23" t="str">
-        <x:v>Wikipedia (inglés): Wilma Mankiller</x:v>
+        <x:v>Wikipedia (English): Wilma Mankiller</x:v>
       </x:c>
       <x:c r="G98" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Wilma_Mankiller</x:v>
@@ -2579,16 +2579,16 @@
         <x:v>Benito Juárez</x:v>
       </x:c>
       <x:c r="C99" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D99" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E99" s="23" t="str">
-        <x:v>México</x:v>
+        <x:v>Mexico</x:v>
       </x:c>
       <x:c r="F99" s="23" t="str">
-        <x:v>Wikipedia (inglés): Benito Juárez</x:v>
+        <x:v>Wikipedia (English): Benito Juárez</x:v>
       </x:c>
       <x:c r="G99" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Benito_Ju%C3%A1rez</x:v>
@@ -2602,16 +2602,16 @@
         <x:v>Elizabeth Peratrovich</x:v>
       </x:c>
       <x:c r="C100" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D100" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E100" s="23" t="str">
         <x:v>Tlingit / Alaska</x:v>
       </x:c>
       <x:c r="F100" s="23" t="str">
-        <x:v>Wikipedia (inglés): Elizabeth Peratrovich</x:v>
+        <x:v>Wikipedia (English): Elizabeth Peratrovich</x:v>
       </x:c>
       <x:c r="G100" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Elizabeth_Peratrovich</x:v>
@@ -2625,16 +2625,16 @@
         <x:v>José Martí</x:v>
       </x:c>
       <x:c r="C101" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D101" s="22" t="str">
-        <x:v>Américas</x:v>
+        <x:v>Americas</x:v>
       </x:c>
       <x:c r="E101" s="23" t="str">
         <x:v>Cuba</x:v>
       </x:c>
       <x:c r="F101" s="23" t="str">
-        <x:v>Wikipedia (inglés): José Martí</x:v>
+        <x:v>Wikipedia (English): José Martí</x:v>
       </x:c>
       <x:c r="G101" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Jos%C3%A9_Mart%C3%AD</x:v>
@@ -2648,16 +2648,16 @@
         <x:v>Wu Zetian</x:v>
       </x:c>
       <x:c r="C102" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D102" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E102" s="23" t="str">
-        <x:v>China / dinastía Zhou</x:v>
+        <x:v>China / Zhou dynasty</x:v>
       </x:c>
       <x:c r="F102" s="23" t="str">
-        <x:v>Wikipedia (inglés): Wu Zetian</x:v>
+        <x:v>Wikipedia (English): Wu Zetian</x:v>
       </x:c>
       <x:c r="G102" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Wu_Zetian</x:v>
@@ -2671,16 +2671,16 @@
         <x:v>Ashoka</x:v>
       </x:c>
       <x:c r="C103" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D103" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E103" s="23" t="str">
-        <x:v>Imperio Maurya</x:v>
+        <x:v>Maurya Empire</x:v>
       </x:c>
       <x:c r="F103" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ashoka</x:v>
+        <x:v>Wikipedia (English): Ashoka</x:v>
       </x:c>
       <x:c r="G103" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ashoka</x:v>
@@ -2691,19 +2691,19 @@
         <x:v>91</x:v>
       </x:c>
       <x:c r="B104" s="23" t="str">
-        <x:v>Emperatriz Suiko</x:v>
+        <x:v>Empress Suiko</x:v>
       </x:c>
       <x:c r="C104" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D104" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E104" s="23" t="str">
-        <x:v>Japón</x:v>
+        <x:v>Japan</x:v>
       </x:c>
       <x:c r="F104" s="23" t="str">
-        <x:v>Wikipedia (inglés): Empress Suiko</x:v>
+        <x:v>Wikipedia (English): Empress Suiko</x:v>
       </x:c>
       <x:c r="G104" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Empress_Suiko</x:v>
@@ -2717,16 +2717,16 @@
         <x:v>Chandragupta Maurya</x:v>
       </x:c>
       <x:c r="C105" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D105" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E105" s="23" t="str">
-        <x:v>Imperio Maurya</x:v>
+        <x:v>Maurya Empire</x:v>
       </x:c>
       <x:c r="F105" s="23" t="str">
-        <x:v>Wikipedia (inglés): Chandragupta Maurya</x:v>
+        <x:v>Wikipedia (English): Chandragupta Maurya</x:v>
       </x:c>
       <x:c r="G105" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Chandragupta_Maurya</x:v>
@@ -2737,19 +2737,19 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="B106" s="23" t="str">
-        <x:v>Emperatriz Genmei</x:v>
+        <x:v>Empress Genmei</x:v>
       </x:c>
       <x:c r="C106" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D106" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E106" s="23" t="str">
-        <x:v>Japón</x:v>
+        <x:v>Japan</x:v>
       </x:c>
       <x:c r="F106" s="23" t="str">
-        <x:v>Wikipedia (inglés): Empress Genmei</x:v>
+        <x:v>Wikipedia (English): Empress Genmei</x:v>
       </x:c>
       <x:c r="G106" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Empress_Genmei</x:v>
@@ -2763,16 +2763,16 @@
         <x:v>Akbar</x:v>
       </x:c>
       <x:c r="C107" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D107" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E107" s="23" t="str">
-        <x:v>Imperio mogol</x:v>
+        <x:v>Mughal Empire</x:v>
       </x:c>
       <x:c r="F107" s="23" t="str">
-        <x:v>Wikipedia (inglés): Akbar</x:v>
+        <x:v>Wikipedia (English): Akbar</x:v>
       </x:c>
       <x:c r="G107" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Akbar</x:v>
@@ -2786,16 +2786,16 @@
         <x:v>Rani Durgavati</x:v>
       </x:c>
       <x:c r="C108" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D108" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E108" s="23" t="str">
-        <x:v>Gondwana / India central</x:v>
+        <x:v>Gondwana / Central India</x:v>
       </x:c>
       <x:c r="F108" s="23" t="str">
-        <x:v>Wikipedia (inglés): Rani Durgavati</x:v>
+        <x:v>Wikipedia (English): Rani Durgavati</x:v>
       </x:c>
       <x:c r="G108" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Rani_Durgavati</x:v>
@@ -2809,16 +2809,16 @@
         <x:v>Babur</x:v>
       </x:c>
       <x:c r="C109" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D109" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E109" s="23" t="str">
-        <x:v>Imperio mogol</x:v>
+        <x:v>Mughal Empire</x:v>
       </x:c>
       <x:c r="F109" s="23" t="str">
-        <x:v>Wikipedia (inglés): Babur</x:v>
+        <x:v>Wikipedia (English): Babur</x:v>
       </x:c>
       <x:c r="G109" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Babur</x:v>
@@ -2832,7 +2832,7 @@
         <x:v>Ahilyabai Holkar</x:v>
       </x:c>
       <x:c r="C110" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D110" s="22" t="str">
         <x:v>Asia</x:v>
@@ -2841,7 +2841,7 @@
         <x:v>Maratha / Malwa</x:v>
       </x:c>
       <x:c r="F110" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ahilyabai Holkar</x:v>
+        <x:v>Wikipedia (English): Ahilyabai Holkar</x:v>
       </x:c>
       <x:c r="G110" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ahilyabai_Holkar</x:v>
@@ -2852,19 +2852,19 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="B111" s="23" t="str">
-        <x:v>Ciro el Grande</x:v>
+        <x:v>Cyrus the Great</x:v>
       </x:c>
       <x:c r="C111" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D111" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E111" s="23" t="str">
-        <x:v>Imperio aqueménida</x:v>
+        <x:v>Achaemenid Empire</x:v>
       </x:c>
       <x:c r="F111" s="23" t="str">
-        <x:v>Wikipedia (inglés): Cyrus the Great</x:v>
+        <x:v>Wikipedia (English): Cyrus the Great</x:v>
       </x:c>
       <x:c r="G111" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Cyrus_the_Great</x:v>
@@ -2878,7 +2878,7 @@
         <x:v>Kittur Chennamma</x:v>
       </x:c>
       <x:c r="C112" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D112" s="22" t="str">
         <x:v>Asia</x:v>
@@ -2887,7 +2887,7 @@
         <x:v>Kittur / India</x:v>
       </x:c>
       <x:c r="F112" s="23" t="str">
-        <x:v>Wikipedia (inglés): Kittur Chennamma</x:v>
+        <x:v>Wikipedia (English): Kittur Chennamma</x:v>
       </x:c>
       <x:c r="G112" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Kittur_Chennamma</x:v>
@@ -2898,19 +2898,19 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B113" s="23" t="str">
-        <x:v>Darío I</x:v>
+        <x:v>Darius the Great</x:v>
       </x:c>
       <x:c r="C113" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D113" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E113" s="23" t="str">
-        <x:v>Imperio aqueménida</x:v>
+        <x:v>Achaemenid Empire</x:v>
       </x:c>
       <x:c r="F113" s="23" t="str">
-        <x:v>Wikipedia (inglés): Darius the Great</x:v>
+        <x:v>Wikipedia (English): Darius the Great</x:v>
       </x:c>
       <x:c r="G113" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Darius_the_Great</x:v>
@@ -2924,7 +2924,7 @@
         <x:v>Rani Lakshmibai</x:v>
       </x:c>
       <x:c r="C114" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D114" s="22" t="str">
         <x:v>Asia</x:v>
@@ -2933,7 +2933,7 @@
         <x:v>Jhansi / India</x:v>
       </x:c>
       <x:c r="F114" s="23" t="str">
-        <x:v>Wikipedia (inglés): Lakshmibai, Rani of Jhansi</x:v>
+        <x:v>Wikipedia (English): Lakshmibai, Rani of Jhansi</x:v>
       </x:c>
       <x:c r="G114" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lakshmibai,_Rani_of_Jhansi</x:v>
@@ -2944,19 +2944,19 @@
         <x:v>102</x:v>
       </x:c>
       <x:c r="B115" s="23" t="str">
-        <x:v>Suleimán el Magnífico</x:v>
+        <x:v>Suleiman the Magnificent</x:v>
       </x:c>
       <x:c r="C115" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D115" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E115" s="23" t="str">
-        <x:v>Imperio otomano</x:v>
+        <x:v>Ottoman Empire</x:v>
       </x:c>
       <x:c r="F115" s="23" t="str">
-        <x:v>Wikipedia (inglés): Suleiman the Magnificent</x:v>
+        <x:v>Wikipedia (English): Suleiman the Magnificent</x:v>
       </x:c>
       <x:c r="G115" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Suleiman_the_Magnificent</x:v>
@@ -2970,16 +2970,16 @@
         <x:v>Cleopatra Thea</x:v>
       </x:c>
       <x:c r="C116" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D116" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E116" s="23" t="str">
-        <x:v>Imperio seléucida</x:v>
+        <x:v>Seleucid Empire</x:v>
       </x:c>
       <x:c r="F116" s="23" t="str">
-        <x:v>Wikipedia (inglés): Cleopatra Thea</x:v>
+        <x:v>Wikipedia (English): Cleopatra Thea</x:v>
       </x:c>
       <x:c r="G116" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Cleopatra_Thea</x:v>
@@ -2990,19 +2990,19 @@
         <x:v>104</x:v>
       </x:c>
       <x:c r="B117" s="23" t="str">
-        <x:v>Saladino</x:v>
+        <x:v>Saladin</x:v>
       </x:c>
       <x:c r="C117" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D117" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E117" s="23" t="str">
-        <x:v>Sultanato ayubí</x:v>
+        <x:v>Ayyubid Sultanate</x:v>
       </x:c>
       <x:c r="F117" s="23" t="str">
-        <x:v>Wikipedia (inglés): Saladin</x:v>
+        <x:v>Wikipedia (English): Saladin</x:v>
       </x:c>
       <x:c r="G117" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Saladin</x:v>
@@ -3016,16 +3016,16 @@
         <x:v>Zenobia</x:v>
       </x:c>
       <x:c r="C118" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D118" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E118" s="23" t="str">
-        <x:v>Palmira</x:v>
+        <x:v>Palmyra</x:v>
       </x:c>
       <x:c r="F118" s="23" t="str">
-        <x:v>Wikipedia (inglés): Zenobia</x:v>
+        <x:v>Wikipedia (English): Zenobia</x:v>
       </x:c>
       <x:c r="G118" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Zenobia</x:v>
@@ -3039,16 +3039,16 @@
         <x:v>Genghis Khan</x:v>
       </x:c>
       <x:c r="C119" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D119" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E119" s="23" t="str">
-        <x:v>Imperio mongol</x:v>
+        <x:v>Mongol Empire</x:v>
       </x:c>
       <x:c r="F119" s="23" t="str">
-        <x:v>Wikipedia (inglés): Genghis Khan</x:v>
+        <x:v>Wikipedia (English): Genghis Khan</x:v>
       </x:c>
       <x:c r="G119" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Genghis_Khan</x:v>
@@ -3062,16 +3062,16 @@
         <x:v>Razia Sultan</x:v>
       </x:c>
       <x:c r="C120" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D120" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E120" s="23" t="str">
-        <x:v>Sultanato de Delhi</x:v>
+        <x:v>Delhi Sultanate</x:v>
       </x:c>
       <x:c r="F120" s="23" t="str">
-        <x:v>Wikipedia (inglés): Razia Sultan</x:v>
+        <x:v>Wikipedia (English): Razia Sultan</x:v>
       </x:c>
       <x:c r="G120" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Razia_Sultan</x:v>
@@ -3085,16 +3085,16 @@
         <x:v>Kublai Khan</x:v>
       </x:c>
       <x:c r="C121" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D121" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E121" s="23" t="str">
-        <x:v>Imperio mongol / Yuan</x:v>
+        <x:v>Mongol Empire / Yuan</x:v>
       </x:c>
       <x:c r="F121" s="23" t="str">
-        <x:v>Wikipedia (inglés): Kublai Khan</x:v>
+        <x:v>Wikipedia (English): Kublai Khan</x:v>
       </x:c>
       <x:c r="G121" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Kublai_Khan</x:v>
@@ -3108,16 +3108,16 @@
         <x:v>Rudrama Devi</x:v>
       </x:c>
       <x:c r="C122" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D122" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E122" s="23" t="str">
-        <x:v>Reino Kakatiya</x:v>
+        <x:v>Kakatiya Kingdom</x:v>
       </x:c>
       <x:c r="F122" s="23" t="str">
-        <x:v>Wikipedia (inglés): Rudrama Devi</x:v>
+        <x:v>Wikipedia (English): Rudrama Devi</x:v>
       </x:c>
       <x:c r="G122" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Rudrama_Devi</x:v>
@@ -3131,16 +3131,16 @@
         <x:v>Tokugawa Ieyasu</x:v>
       </x:c>
       <x:c r="C123" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D123" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E123" s="23" t="str">
-        <x:v>Japón</x:v>
+        <x:v>Japan</x:v>
       </x:c>
       <x:c r="F123" s="23" t="str">
-        <x:v>Wikipedia (inglés): Tokugawa Ieyasu</x:v>
+        <x:v>Wikipedia (English): Tokugawa Ieyasu</x:v>
       </x:c>
       <x:c r="G123" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tokugawa_Ieyasu</x:v>
@@ -3151,19 +3151,19 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B124" s="23" t="str">
-        <x:v>Rani Abbakka Chowta</x:v>
+        <x:v>Abbakka Chowta</x:v>
       </x:c>
       <x:c r="C124" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D124" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E124" s="23" t="str">
-        <x:v>Ullal / costa de Karnataka</x:v>
+        <x:v>Ullal / Karnataka coast</x:v>
       </x:c>
       <x:c r="F124" s="23" t="str">
-        <x:v>Wikipedia (inglés): Abbakka Chowta</x:v>
+        <x:v>Wikipedia (English): Abbakka Chowta</x:v>
       </x:c>
       <x:c r="G124" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Abbakka_Chowta</x:v>
@@ -3177,7 +3177,7 @@
         <x:v>Qin Shi Huang</x:v>
       </x:c>
       <x:c r="C125" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D125" s="22" t="str">
         <x:v>Asia</x:v>
@@ -3186,7 +3186,7 @@
         <x:v>China</x:v>
       </x:c>
       <x:c r="F125" s="23" t="str">
-        <x:v>Wikipedia (inglés): Qin Shi Huang</x:v>
+        <x:v>Wikipedia (English): Qin Shi Huang</x:v>
       </x:c>
       <x:c r="G125" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Qin_Shi_Huang</x:v>
@@ -3197,19 +3197,19 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="B126" s="23" t="str">
-        <x:v>Tarabai Bhonsle</x:v>
+        <x:v>Tarabai</x:v>
       </x:c>
       <x:c r="C126" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D126" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E126" s="23" t="str">
-        <x:v>Imperio Maratha</x:v>
+        <x:v>Maratha Empire</x:v>
       </x:c>
       <x:c r="F126" s="23" t="str">
-        <x:v>Wikipedia (inglés): Tarabai</x:v>
+        <x:v>Wikipedia (English): Tarabai</x:v>
       </x:c>
       <x:c r="G126" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tarabai</x:v>
@@ -3220,19 +3220,19 @@
         <x:v>114</x:v>
       </x:c>
       <x:c r="B127" s="23" t="str">
-        <x:v>Sejong el Grande</x:v>
+        <x:v>Sejong the Great</x:v>
       </x:c>
       <x:c r="C127" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D127" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E127" s="23" t="str">
-        <x:v>Joseon / Corea</x:v>
+        <x:v>Joseon / Korea</x:v>
       </x:c>
       <x:c r="F127" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sejong the Great</x:v>
+        <x:v>Wikipedia (English): Sejong the Great</x:v>
       </x:c>
       <x:c r="G127" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sejong_the_Great</x:v>
@@ -3246,16 +3246,16 @@
         <x:v>Chand Bibi</x:v>
       </x:c>
       <x:c r="C128" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D128" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E128" s="23" t="str">
-        <x:v>Ahmednagar y Bijapur</x:v>
+        <x:v>Ahmadnagar and Bijapur</x:v>
       </x:c>
       <x:c r="F128" s="23" t="str">
-        <x:v>Wikipedia (inglés): Chand Bibi</x:v>
+        <x:v>Wikipedia (English): Chand Bibi</x:v>
       </x:c>
       <x:c r="G128" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Chand_Bibi</x:v>
@@ -3269,16 +3269,16 @@
         <x:v>Suryavarman II</x:v>
       </x:c>
       <x:c r="C129" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D129" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E129" s="23" t="str">
-        <x:v>Imperio jemer</x:v>
+        <x:v>Khmer Empire</x:v>
       </x:c>
       <x:c r="F129" s="23" t="str">
-        <x:v>Wikipedia (inglés): Suryavarman II</x:v>
+        <x:v>Wikipedia (English): Suryavarman II</x:v>
       </x:c>
       <x:c r="G129" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Suryavarman_II</x:v>
@@ -3292,16 +3292,16 @@
         <x:v>Didda</x:v>
       </x:c>
       <x:c r="C130" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D130" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E130" s="23" t="str">
-        <x:v>Cachemira</x:v>
+        <x:v>Kashmir</x:v>
       </x:c>
       <x:c r="F130" s="23" t="str">
-        <x:v>Wikipedia (inglés): Didda</x:v>
+        <x:v>Wikipedia (English): Didda</x:v>
       </x:c>
       <x:c r="G130" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Didda</x:v>
@@ -3315,16 +3315,16 @@
         <x:v>Jayavarman VII</x:v>
       </x:c>
       <x:c r="C131" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D131" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E131" s="23" t="str">
-        <x:v>Imperio jemer</x:v>
+        <x:v>Khmer Empire</x:v>
       </x:c>
       <x:c r="F131" s="23" t="str">
-        <x:v>Wikipedia (inglés): Jayavarman VII</x:v>
+        <x:v>Wikipedia (English): Jayavarman VII</x:v>
       </x:c>
       <x:c r="G131" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Jayavarman_VII</x:v>
@@ -3335,19 +3335,19 @@
         <x:v>119</x:v>
       </x:c>
       <x:c r="B132" s="23" t="str">
-        <x:v>Seondeok de Silla</x:v>
+        <x:v>Queen Seondeok of Silla</x:v>
       </x:c>
       <x:c r="C132" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D132" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E132" s="23" t="str">
-        <x:v>Reino de Silla / Corea</x:v>
+        <x:v>Silla Kingdom / Korea</x:v>
       </x:c>
       <x:c r="F132" s="23" t="str">
-        <x:v>Wikipedia (inglés): Queen Seondeok of Silla</x:v>
+        <x:v>Wikipedia (English): Queen Seondeok of Silla</x:v>
       </x:c>
       <x:c r="G132" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Queen_Seondeok_of_Silla</x:v>
@@ -3361,16 +3361,16 @@
         <x:v>Bayinnaung</x:v>
       </x:c>
       <x:c r="C133" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D133" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E133" s="23" t="str">
-        <x:v>Imperio Toungoo / Birmania</x:v>
+        <x:v>Toungoo Empire / Burma</x:v>
       </x:c>
       <x:c r="F133" s="23" t="str">
-        <x:v>Wikipedia (inglés): Bayinnaung</x:v>
+        <x:v>Wikipedia (English): Bayinnaung</x:v>
       </x:c>
       <x:c r="G133" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Bayinnaung</x:v>
@@ -3381,19 +3381,19 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="B134" s="23" t="str">
-        <x:v>Lü Zhi</x:v>
+        <x:v>Empress Lü</x:v>
       </x:c>
       <x:c r="C134" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D134" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E134" s="23" t="str">
-        <x:v>China / dinastía Han</x:v>
+        <x:v>China / Han dynasty</x:v>
       </x:c>
       <x:c r="F134" s="23" t="str">
-        <x:v>Wikipedia (inglés): Empress Lü</x:v>
+        <x:v>Wikipedia (English): Empress Lü</x:v>
       </x:c>
       <x:c r="G134" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Empress_L%C3%BC</x:v>
@@ -3404,19 +3404,19 @@
         <x:v>122</x:v>
       </x:c>
       <x:c r="B135" s="23" t="str">
-        <x:v>Harún al-Rashid</x:v>
+        <x:v>Harun al-Rashid</x:v>
       </x:c>
       <x:c r="C135" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D135" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E135" s="23" t="str">
-        <x:v>Califato abasí</x:v>
+        <x:v>Abbasid Caliphate</x:v>
       </x:c>
       <x:c r="F135" s="23" t="str">
-        <x:v>Wikipedia (inglés): Harun al-Rashid</x:v>
+        <x:v>Wikipedia (English): Harun al-Rashid</x:v>
       </x:c>
       <x:c r="G135" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Harun_al-Rashid</x:v>
@@ -3430,7 +3430,7 @@
         <x:v>Lady Triệu</x:v>
       </x:c>
       <x:c r="C136" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D136" s="22" t="str">
         <x:v>Asia</x:v>
@@ -3439,7 +3439,7 @@
         <x:v>Vietnam</x:v>
       </x:c>
       <x:c r="F136" s="23" t="str">
-        <x:v>Wikipedia (inglés): Lady Triệu</x:v>
+        <x:v>Wikipedia (English): Lady Triệu</x:v>
       </x:c>
       <x:c r="G136" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lady_Tri%E1%BB%87u</x:v>
@@ -3453,16 +3453,16 @@
         <x:v>Hammurabi</x:v>
       </x:c>
       <x:c r="C137" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D137" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E137" s="23" t="str">
-        <x:v>Babilonia</x:v>
+        <x:v>Babylon</x:v>
       </x:c>
       <x:c r="F137" s="23" t="str">
-        <x:v>Wikipedia (inglés): Hammurabi</x:v>
+        <x:v>Wikipedia (English): Hammurabi</x:v>
       </x:c>
       <x:c r="G137" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Hammurabi</x:v>
@@ -3473,10 +3473,10 @@
         <x:v>125</x:v>
       </x:c>
       <x:c r="B138" s="23" t="str">
-        <x:v>Trưng Trắc</x:v>
+        <x:v>Trưng Nhị</x:v>
       </x:c>
       <x:c r="C138" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D138" s="22" t="str">
         <x:v>Asia</x:v>
@@ -3485,7 +3485,7 @@
         <x:v>Vietnam</x:v>
       </x:c>
       <x:c r="F138" s="23" t="str">
-        <x:v>Wikipedia (inglés): Trưng sisters</x:v>
+        <x:v>Wikipedia (English): Trưng sisters</x:v>
       </x:c>
       <x:c r="G138" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tr%C6%B0ng_sisters</x:v>
@@ -3496,19 +3496,19 @@
         <x:v>126</x:v>
       </x:c>
       <x:c r="B139" s="23" t="str">
-        <x:v>Asurbanipal</x:v>
+        <x:v>Ashurbanipal</x:v>
       </x:c>
       <x:c r="C139" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D139" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E139" s="23" t="str">
-        <x:v>Imperio neoasirio</x:v>
+        <x:v>Neo-Assyrian Empire</x:v>
       </x:c>
       <x:c r="F139" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ashurbanipal</x:v>
+        <x:v>Wikipedia (English): Ashurbanipal</x:v>
       </x:c>
       <x:c r="G139" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ashurbanipal</x:v>
@@ -3522,7 +3522,7 @@
         <x:v>Trưng Nhị</x:v>
       </x:c>
       <x:c r="C140" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D140" s="22" t="str">
         <x:v>Asia</x:v>
@@ -3531,7 +3531,7 @@
         <x:v>Vietnam</x:v>
       </x:c>
       <x:c r="F140" s="23" t="str">
-        <x:v>Wikipedia (inglés): Trưng sisters</x:v>
+        <x:v>Wikipedia (English): Trưng sisters</x:v>
       </x:c>
       <x:c r="G140" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tr%C6%B0ng_sisters</x:v>
@@ -3545,16 +3545,16 @@
         <x:v>Rajaraja I</x:v>
       </x:c>
       <x:c r="C141" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D141" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E141" s="23" t="str">
-        <x:v>Imperio Chola</x:v>
+        <x:v>Chola Empire</x:v>
       </x:c>
       <x:c r="F141" s="23" t="str">
-        <x:v>Wikipedia (inglés): Rajaraja I</x:v>
+        <x:v>Wikipedia (English): Rajaraja I</x:v>
       </x:c>
       <x:c r="G141" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Rajaraja_I</x:v>
@@ -3568,16 +3568,16 @@
         <x:v>Suriyothai</x:v>
       </x:c>
       <x:c r="C142" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D142" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E142" s="23" t="str">
-        <x:v>Ayutthaya / Tailandia</x:v>
+        <x:v>Ayutthaya / Thailand</x:v>
       </x:c>
       <x:c r="F142" s="23" t="str">
-        <x:v>Wikipedia (inglés): Suriyothai</x:v>
+        <x:v>Wikipedia (English): Suriyothai</x:v>
       </x:c>
       <x:c r="G142" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Suriyothai</x:v>
@@ -3591,16 +3591,16 @@
         <x:v>Ranjit Singh</x:v>
       </x:c>
       <x:c r="C143" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D143" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E143" s="23" t="str">
-        <x:v>Imperio sij</x:v>
+        <x:v>Sikh Empire</x:v>
       </x:c>
       <x:c r="F143" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ranjit Singh</x:v>
+        <x:v>Wikipedia (English): Ranjit Singh</x:v>
       </x:c>
       <x:c r="G143" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ranjit_Singh</x:v>
@@ -3614,7 +3614,7 @@
         <x:v>Tribhuwana Wijayatunggadewi</x:v>
       </x:c>
       <x:c r="C144" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D144" s="22" t="str">
         <x:v>Asia</x:v>
@@ -3623,7 +3623,7 @@
         <x:v>Majapahit / Java</x:v>
       </x:c>
       <x:c r="F144" s="23" t="str">
-        <x:v>Wikipedia (inglés): Tribhuwana Wijayatunggadewi</x:v>
+        <x:v>Wikipedia (English): Tribhuwana Wijayatunggadewi</x:v>
       </x:c>
       <x:c r="G144" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tribhuwana_Wijayatunggadewi</x:v>
@@ -3637,16 +3637,16 @@
         <x:v>Prithvi Narayan Shah</x:v>
       </x:c>
       <x:c r="C145" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D145" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E145" s="23" t="str">
-        <x:v>Reino de Gorkha / Nepal</x:v>
+        <x:v>Gorkha Kingdom / Nepal</x:v>
       </x:c>
       <x:c r="F145" s="23" t="str">
-        <x:v>Wikipedia (inglés): Prithvi Narayan Shah</x:v>
+        <x:v>Wikipedia (English): Prithvi Narayan Shah</x:v>
       </x:c>
       <x:c r="G145" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Prithvi_Narayan_Shah</x:v>
@@ -3660,16 +3660,16 @@
         <x:v>Töregene Khatun</x:v>
       </x:c>
       <x:c r="C146" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D146" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E146" s="23" t="str">
-        <x:v>Imperio mongol</x:v>
+        <x:v>Mongol Empire</x:v>
       </x:c>
       <x:c r="F146" s="23" t="str">
-        <x:v>Wikipedia (inglés): Töregene Khatun</x:v>
+        <x:v>Wikipedia (English): Töregene Khatun</x:v>
       </x:c>
       <x:c r="G146" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/T%C3%B6regene_Khatun</x:v>
@@ -3683,16 +3683,16 @@
         <x:v>Tipu Sultan</x:v>
       </x:c>
       <x:c r="C147" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D147" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E147" s="23" t="str">
-        <x:v>Reino de Mysore</x:v>
+        <x:v>Kingdom of Mysore</x:v>
       </x:c>
       <x:c r="F147" s="23" t="str">
-        <x:v>Wikipedia (inglés): Tipu Sultan</x:v>
+        <x:v>Wikipedia (English): Tipu Sultan</x:v>
       </x:c>
       <x:c r="G147" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Tipu_Sultan</x:v>
@@ -3703,10 +3703,10 @@
         <x:v>135</x:v>
       </x:c>
       <x:c r="B148" s="23" t="str">
-        <x:v>Mandukhai Khatun</x:v>
+        <x:v>Mandukhai</x:v>
       </x:c>
       <x:c r="C148" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D148" s="22" t="str">
         <x:v>Asia</x:v>
@@ -3715,7 +3715,7 @@
         <x:v>Mongolia</x:v>
       </x:c>
       <x:c r="F148" s="23" t="str">
-        <x:v>Wikipedia (inglés): Mandukhai</x:v>
+        <x:v>Wikipedia (English): Mandukhai</x:v>
       </x:c>
       <x:c r="G148" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Mandukhai</x:v>
@@ -3729,16 +3729,16 @@
         <x:v>Shivaji</x:v>
       </x:c>
       <x:c r="C149" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D149" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E149" s="23" t="str">
-        <x:v>Imperio Maratha</x:v>
+        <x:v>Maratha Empire</x:v>
       </x:c>
       <x:c r="F149" s="23" t="str">
-        <x:v>Wikipedia (inglés): Shivaji</x:v>
+        <x:v>Wikipedia (English): Shivaji</x:v>
       </x:c>
       <x:c r="G149" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Shivaji</x:v>
@@ -3752,16 +3752,16 @@
         <x:v>Sorghaghtani Beki</x:v>
       </x:c>
       <x:c r="C150" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D150" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E150" s="23" t="str">
-        <x:v>Imperio mongol</x:v>
+        <x:v>Mongol Empire</x:v>
       </x:c>
       <x:c r="F150" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sorghaghtani Beki</x:v>
+        <x:v>Wikipedia (English): Sorghaghtani Beki</x:v>
       </x:c>
       <x:c r="G150" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sorghaghtani_Beki</x:v>
@@ -3775,16 +3775,16 @@
         <x:v>Mustafa Kemal Atatürk</x:v>
       </x:c>
       <x:c r="C151" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D151" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E151" s="23" t="str">
-        <x:v>Turquía</x:v>
+        <x:v>Turkey</x:v>
       </x:c>
       <x:c r="F151" s="23" t="str">
-        <x:v>Wikipedia (inglés): Mustafa Kemal Atatürk</x:v>
+        <x:v>Wikipedia (English): Mustafa Kemal Atatürk</x:v>
       </x:c>
       <x:c r="G151" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Mustafa_Kemal_Atat%C3%BCrk</x:v>
@@ -3798,16 +3798,16 @@
         <x:v>Nur Jahan</x:v>
       </x:c>
       <x:c r="C152" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D152" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E152" s="23" t="str">
-        <x:v>Imperio mogol</x:v>
+        <x:v>Mughal Empire</x:v>
       </x:c>
       <x:c r="F152" s="23" t="str">
-        <x:v>Wikipedia (inglés): Nur Jahan</x:v>
+        <x:v>Wikipedia (English): Nur Jahan</x:v>
       </x:c>
       <x:c r="G152" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Nur_Jahan</x:v>
@@ -3821,16 +3821,16 @@
         <x:v>Timur</x:v>
       </x:c>
       <x:c r="C153" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D153" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E153" s="23" t="str">
-        <x:v>Imperio timúrida</x:v>
+        <x:v>Timurid Empire</x:v>
       </x:c>
       <x:c r="F153" s="23" t="str">
-        <x:v>Wikipedia (inglés): Timur</x:v>
+        <x:v>Wikipedia (English): Timur</x:v>
       </x:c>
       <x:c r="G153" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Timur</x:v>
@@ -3841,19 +3841,19 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="B154" s="23" t="str">
-        <x:v>Emperatriz viuda Cixi</x:v>
+        <x:v>Empress Dowager Cixi</x:v>
       </x:c>
       <x:c r="C154" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D154" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E154" s="23" t="str">
-        <x:v>China / dinastía Qing</x:v>
+        <x:v>China / Qing dynasty</x:v>
       </x:c>
       <x:c r="F154" s="23" t="str">
-        <x:v>Wikipedia (inglés): Empress Dowager Cixi</x:v>
+        <x:v>Wikipedia (English): Empress Dowager Cixi</x:v>
       </x:c>
       <x:c r="G154" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Empress_Dowager_Cixi</x:v>
@@ -3864,19 +3864,19 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="B155" s="23" t="str">
-        <x:v>Zhu Yuanzhang</x:v>
+        <x:v>Hongwu Emperor</x:v>
       </x:c>
       <x:c r="C155" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D155" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E155" s="23" t="str">
-        <x:v>China / dinastía Ming</x:v>
+        <x:v>China / Ming dynasty</x:v>
       </x:c>
       <x:c r="F155" s="23" t="str">
-        <x:v>Wikipedia (inglés): Hongwu Emperor</x:v>
+        <x:v>Wikipedia (English): Hongwu Emperor</x:v>
       </x:c>
       <x:c r="G155" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Hongwu_Emperor</x:v>
@@ -3887,19 +3887,19 @@
         <x:v>143</x:v>
       </x:c>
       <x:c r="B156" s="23" t="str">
-        <x:v>Sultanah Safiatuddin</x:v>
+        <x:v>Taj ul-Alam</x:v>
       </x:c>
       <x:c r="C156" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D156" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E156" s="23" t="str">
-        <x:v>Sultanato de Aceh</x:v>
+        <x:v>Sultanate of Aceh</x:v>
       </x:c>
       <x:c r="F156" s="23" t="str">
-        <x:v>Wikipedia (inglés): Taj ul-Alam</x:v>
+        <x:v>Wikipedia (English): Taj ul-Alam</x:v>
       </x:c>
       <x:c r="G156" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Taj_ul-Alam</x:v>
@@ -3913,16 +3913,16 @@
         <x:v>Kanishka</x:v>
       </x:c>
       <x:c r="C157" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D157" s="22" t="str">
         <x:v>Asia</x:v>
       </x:c>
       <x:c r="E157" s="23" t="str">
-        <x:v>Imperio kushán</x:v>
+        <x:v>Kushan Empire</x:v>
       </x:c>
       <x:c r="F157" s="23" t="str">
-        <x:v>Wikipedia (inglés): Kanishka</x:v>
+        <x:v>Wikipedia (English): Kanishka</x:v>
       </x:c>
       <x:c r="G157" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Kanishka</x:v>
@@ -3936,16 +3936,16 @@
         <x:v>Boudica</x:v>
       </x:c>
       <x:c r="C158" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D158" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E158" s="23" t="str">
-        <x:v>Iceni / Britania</x:v>
+        <x:v>Iceni / Britannia</x:v>
       </x:c>
       <x:c r="F158" s="23" t="str">
-        <x:v>Wikipedia (inglés): Boudica</x:v>
+        <x:v>Wikipedia (English): Boudica</x:v>
       </x:c>
       <x:c r="G158" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Boudica</x:v>
@@ -3956,19 +3956,19 @@
         <x:v>146</x:v>
       </x:c>
       <x:c r="B159" s="23" t="str">
-        <x:v>Alejandro Magno</x:v>
+        <x:v>Alexander the Great</x:v>
       </x:c>
       <x:c r="C159" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D159" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E159" s="23" t="str">
-        <x:v>Macedonia antigua</x:v>
+        <x:v>Macedon</x:v>
       </x:c>
       <x:c r="F159" s="23" t="str">
-        <x:v>Wikipedia (inglés): Alexander the Great</x:v>
+        <x:v>Wikipedia (English): Alexander the Great</x:v>
       </x:c>
       <x:c r="G159" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Alexander_the_Great</x:v>
@@ -3979,19 +3979,19 @@
         <x:v>147</x:v>
       </x:c>
       <x:c r="B160" s="23" t="str">
-        <x:v>Olga de Kiev</x:v>
+        <x:v>Olga of Kiev</x:v>
       </x:c>
       <x:c r="C160" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D160" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E160" s="23" t="str">
-        <x:v>Rus de Kiev</x:v>
+        <x:v>Kievan Rus'</x:v>
       </x:c>
       <x:c r="F160" s="23" t="str">
-        <x:v>Wikipedia (inglés): Olga of Kiev</x:v>
+        <x:v>Wikipedia (English): Olga of Kiev</x:v>
       </x:c>
       <x:c r="G160" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Olga_of_Kiev</x:v>
@@ -4002,19 +4002,19 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="B161" s="23" t="str">
-        <x:v>Julio César</x:v>
+        <x:v>Julius Caesar</x:v>
       </x:c>
       <x:c r="C161" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D161" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E161" s="23" t="str">
-        <x:v>República romana</x:v>
+        <x:v>Roman Republic</x:v>
       </x:c>
       <x:c r="F161" s="23" t="str">
-        <x:v>Wikipedia (inglés): Julius Caesar</x:v>
+        <x:v>Wikipedia (English): Julius Caesar</x:v>
       </x:c>
       <x:c r="G161" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Julius_Caesar</x:v>
@@ -4025,19 +4025,19 @@
         <x:v>149</x:v>
       </x:c>
       <x:c r="B162" s="23" t="str">
-        <x:v>Leonor de Aquitania</x:v>
+        <x:v>Eleanor of Aquitaine</x:v>
       </x:c>
       <x:c r="C162" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D162" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E162" s="23" t="str">
-        <x:v>Aquitania / Francia</x:v>
+        <x:v>Aquitaine / France</x:v>
       </x:c>
       <x:c r="F162" s="23" t="str">
-        <x:v>Wikipedia (inglés): Eleanor of Aquitaine</x:v>
+        <x:v>Wikipedia (English): Eleanor of Aquitaine</x:v>
       </x:c>
       <x:c r="G162" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Eleanor_of_Aquitaine</x:v>
@@ -4048,19 +4048,19 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="B163" s="23" t="str">
-        <x:v>Carlomagno</x:v>
+        <x:v>Charlemagne</x:v>
       </x:c>
       <x:c r="C163" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D163" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E163" s="23" t="str">
-        <x:v>Imperio carolingio</x:v>
+        <x:v>Carolingian Empire</x:v>
       </x:c>
       <x:c r="F163" s="23" t="str">
-        <x:v>Wikipedia (inglés): Charlemagne</x:v>
+        <x:v>Wikipedia (English): Charlemagne</x:v>
       </x:c>
       <x:c r="G163" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Charlemagne</x:v>
@@ -4071,19 +4071,19 @@
         <x:v>151</x:v>
       </x:c>
       <x:c r="B164" s="23" t="str">
-        <x:v>Isabel I de Castilla</x:v>
+        <x:v>Isabella I of Castile</x:v>
       </x:c>
       <x:c r="C164" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D164" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E164" s="23" t="str">
-        <x:v>Castilla / España</x:v>
+        <x:v>Castile / Spain</x:v>
       </x:c>
       <x:c r="F164" s="23" t="str">
-        <x:v>Wikipedia (inglés): Isabella I of Castile</x:v>
+        <x:v>Wikipedia (English): Isabella I of Castile</x:v>
       </x:c>
       <x:c r="G164" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Isabella_I_of_Castile</x:v>
@@ -4094,19 +4094,19 @@
         <x:v>152</x:v>
       </x:c>
       <x:c r="B165" s="23" t="str">
-        <x:v>Alfredo el Grande</x:v>
+        <x:v>Alfred the Great</x:v>
       </x:c>
       <x:c r="C165" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D165" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E165" s="23" t="str">
-        <x:v>Wessex / Inglaterra</x:v>
+        <x:v>Wessex / England</x:v>
       </x:c>
       <x:c r="F165" s="23" t="str">
-        <x:v>Wikipedia (inglés): Alfred the Great</x:v>
+        <x:v>Wikipedia (English): Alfred the Great</x:v>
       </x:c>
       <x:c r="G165" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Alfred_the_Great</x:v>
@@ -4117,19 +4117,19 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="B166" s="23" t="str">
-        <x:v>Isabel I de Inglaterra</x:v>
+        <x:v>Elizabeth I</x:v>
       </x:c>
       <x:c r="C166" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D166" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E166" s="23" t="str">
-        <x:v>Inglaterra</x:v>
+        <x:v>England</x:v>
       </x:c>
       <x:c r="F166" s="23" t="str">
-        <x:v>Wikipedia (inglés): Elizabeth I</x:v>
+        <x:v>Wikipedia (English): Elizabeth I</x:v>
       </x:c>
       <x:c r="G166" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Elizabeth_I</x:v>
@@ -4140,19 +4140,19 @@
         <x:v>154</x:v>
       </x:c>
       <x:c r="B167" s="23" t="str">
-        <x:v>Guillermo el Conquistador</x:v>
+        <x:v>William the Conqueror</x:v>
       </x:c>
       <x:c r="C167" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D167" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E167" s="23" t="str">
-        <x:v>Normandía e Inglaterra</x:v>
+        <x:v>Normandy and England</x:v>
       </x:c>
       <x:c r="F167" s="23" t="str">
-        <x:v>Wikipedia (inglés): William the Conqueror</x:v>
+        <x:v>Wikipedia (English): William the Conqueror</x:v>
       </x:c>
       <x:c r="G167" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/William_the_Conqueror</x:v>
@@ -4163,19 +4163,19 @@
         <x:v>155</x:v>
       </x:c>
       <x:c r="B168" s="23" t="str">
-        <x:v>Catalina la Grande</x:v>
+        <x:v>Catherine the Great</x:v>
       </x:c>
       <x:c r="C168" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D168" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E168" s="23" t="str">
-        <x:v>Imperio ruso</x:v>
+        <x:v>Russian Empire</x:v>
       </x:c>
       <x:c r="F168" s="23" t="str">
-        <x:v>Wikipedia (inglés): Catherine the Great</x:v>
+        <x:v>Wikipedia (English): Catherine the Great</x:v>
       </x:c>
       <x:c r="G168" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Catherine_the_Great</x:v>
@@ -4186,19 +4186,19 @@
         <x:v>156</x:v>
       </x:c>
       <x:c r="B169" s="23" t="str">
-        <x:v>Napoleón Bonaparte</x:v>
+        <x:v>Napoleon</x:v>
       </x:c>
       <x:c r="C169" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D169" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E169" s="23" t="str">
-        <x:v>Francia</x:v>
+        <x:v>French Empire</x:v>
       </x:c>
       <x:c r="F169" s="23" t="str">
-        <x:v>Wikipedia (inglés): Napoleon</x:v>
+        <x:v>Wikipedia (English): Napoleon</x:v>
       </x:c>
       <x:c r="G169" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Napoleon</x:v>
@@ -4209,19 +4209,19 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="B170" s="23" t="str">
-        <x:v>María Teresa de Austria</x:v>
+        <x:v>Maria Theresa</x:v>
       </x:c>
       <x:c r="C170" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D170" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E170" s="23" t="str">
-        <x:v>Monarquía de los Habsburgo</x:v>
+        <x:v>Habsburg Monarchy</x:v>
       </x:c>
       <x:c r="F170" s="23" t="str">
-        <x:v>Wikipedia (inglés): Maria Theresa</x:v>
+        <x:v>Wikipedia (English): Maria Theresa</x:v>
       </x:c>
       <x:c r="G170" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Maria_Theresa</x:v>
@@ -4232,19 +4232,19 @@
         <x:v>158</x:v>
       </x:c>
       <x:c r="B171" s="23" t="str">
-        <x:v>Pedro el Grande</x:v>
+        <x:v>Peter the Great</x:v>
       </x:c>
       <x:c r="C171" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D171" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E171" s="23" t="str">
-        <x:v>Rusia</x:v>
+        <x:v>Russia</x:v>
       </x:c>
       <x:c r="F171" s="23" t="str">
-        <x:v>Wikipedia (inglés): Peter the Great</x:v>
+        <x:v>Wikipedia (English): Peter the Great</x:v>
       </x:c>
       <x:c r="G171" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Peter_the_Great</x:v>
@@ -4255,19 +4255,19 @@
         <x:v>159</x:v>
       </x:c>
       <x:c r="B172" s="23" t="str">
-        <x:v>Margarita I de Dinamarca</x:v>
+        <x:v>Margaret I of Denmark</x:v>
       </x:c>
       <x:c r="C172" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D172" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E172" s="23" t="str">
-        <x:v>Unión de Kalmar</x:v>
+        <x:v>Kalmar Union</x:v>
       </x:c>
       <x:c r="F172" s="23" t="str">
-        <x:v>Wikipedia (inglés): Margaret I of Denmark</x:v>
+        <x:v>Wikipedia (English): Margaret I of Denmark</x:v>
       </x:c>
       <x:c r="G172" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Margaret_I_of_Denmark</x:v>
@@ -4278,19 +4278,19 @@
         <x:v>160</x:v>
       </x:c>
       <x:c r="B173" s="23" t="str">
-        <x:v>Iván IV de Rusia</x:v>
+        <x:v>Ivan the Terrible</x:v>
       </x:c>
       <x:c r="C173" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D173" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E173" s="23" t="str">
-        <x:v>Rusia</x:v>
+        <x:v>Russia</x:v>
       </x:c>
       <x:c r="F173" s="23" t="str">
-        <x:v>Wikipedia (inglés): Ivan the Terrible</x:v>
+        <x:v>Wikipedia (English): Ivan the Terrible</x:v>
       </x:c>
       <x:c r="G173" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ivan_the_Terrible</x:v>
@@ -4301,19 +4301,19 @@
         <x:v>161</x:v>
       </x:c>
       <x:c r="B174" s="23" t="str">
-        <x:v>Irene de Atenas</x:v>
+        <x:v>Irene of Athens</x:v>
       </x:c>
       <x:c r="C174" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D174" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E174" s="23" t="str">
-        <x:v>Imperio bizantino</x:v>
+        <x:v>Byzantine Empire</x:v>
       </x:c>
       <x:c r="F174" s="23" t="str">
-        <x:v>Wikipedia (inglés): Irene of Athens</x:v>
+        <x:v>Wikipedia (English): Irene of Athens</x:v>
       </x:c>
       <x:c r="G174" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Irene_of_Athens</x:v>
@@ -4327,16 +4327,16 @@
         <x:v>Skanderbeg</x:v>
       </x:c>
       <x:c r="C175" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D175" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E175" s="23" t="str">
         <x:v>Albania</x:v>
       </x:c>
       <x:c r="F175" s="23" t="str">
-        <x:v>Wikipedia (inglés): Skanderbeg</x:v>
+        <x:v>Wikipedia (English): Skanderbeg</x:v>
       </x:c>
       <x:c r="G175" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Skanderbeg</x:v>
@@ -4350,16 +4350,16 @@
         <x:v>Teodora</x:v>
       </x:c>
       <x:c r="C176" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D176" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E176" s="23" t="str">
-        <x:v>Imperio bizantino</x:v>
+        <x:v>Byzantine Empire</x:v>
       </x:c>
       <x:c r="F176" s="23" t="str">
-        <x:v>Wikipedia (inglés): Theodora (wife of Justinian I)</x:v>
+        <x:v>Wikipedia (English): Theodora (wife of Justinian I)</x:v>
       </x:c>
       <x:c r="G176" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Theodora_(wife_of_Justinian_I)</x:v>
@@ -4370,19 +4370,19 @@
         <x:v>164</x:v>
       </x:c>
       <x:c r="B177" s="23" t="str">
-        <x:v>Juan III Sobieski</x:v>
+        <x:v>John III Sobieski</x:v>
       </x:c>
       <x:c r="C177" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D177" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E177" s="23" t="str">
-        <x:v>Polonia-Lituania</x:v>
+        <x:v>Poland-Lithuania</x:v>
       </x:c>
       <x:c r="F177" s="23" t="str">
-        <x:v>Wikipedia (inglés): John III Sobieski</x:v>
+        <x:v>Wikipedia (English): John III Sobieski</x:v>
       </x:c>
       <x:c r="G177" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/John_III_Sobieski</x:v>
@@ -4393,19 +4393,19 @@
         <x:v>165</x:v>
       </x:c>
       <x:c r="B178" s="23" t="str">
-        <x:v>Amalasunta</x:v>
+        <x:v>Amalasuintha</x:v>
       </x:c>
       <x:c r="C178" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D178" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E178" s="23" t="str">
-        <x:v>Reino ostrogodo / Italia</x:v>
+        <x:v>Ostrogothic Kingdom / Italy</x:v>
       </x:c>
       <x:c r="F178" s="23" t="str">
-        <x:v>Wikipedia (inglés): Amalasuintha</x:v>
+        <x:v>Wikipedia (English): Amalasuintha</x:v>
       </x:c>
       <x:c r="G178" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Amalasuintha</x:v>
@@ -4416,19 +4416,19 @@
         <x:v>166</x:v>
       </x:c>
       <x:c r="B179" s="23" t="str">
-        <x:v>Gustavo II Adolfo</x:v>
+        <x:v>Gustavus Adolphus</x:v>
       </x:c>
       <x:c r="C179" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D179" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E179" s="23" t="str">
-        <x:v>Suecia</x:v>
+        <x:v>Sweden</x:v>
       </x:c>
       <x:c r="F179" s="23" t="str">
-        <x:v>Wikipedia (inglés): Gustavus Adolphus</x:v>
+        <x:v>Wikipedia (English): Gustavus Adolphus</x:v>
       </x:c>
       <x:c r="G179" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Gustavus_Adolphus</x:v>
@@ -4439,19 +4439,19 @@
         <x:v>167</x:v>
       </x:c>
       <x:c r="B180" s="23" t="str">
-        <x:v>Brunilda de Austrasia</x:v>
+        <x:v>Brunhilda of Austrasia</x:v>
       </x:c>
       <x:c r="C180" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D180" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E180" s="23" t="str">
-        <x:v>Austrasia / francos</x:v>
+        <x:v>Austrasia / Franks</x:v>
       </x:c>
       <x:c r="F180" s="23" t="str">
-        <x:v>Wikipedia (inglés): Brunhilda of Austrasia</x:v>
+        <x:v>Wikipedia (English): Brunhilda of Austrasia</x:v>
       </x:c>
       <x:c r="G180" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Brunhilda_of_Austrasia</x:v>
@@ -4465,16 +4465,16 @@
         <x:v>Harald Bluetooth</x:v>
       </x:c>
       <x:c r="C181" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D181" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E181" s="23" t="str">
-        <x:v>Dinamarca</x:v>
+        <x:v>Denmark</x:v>
       </x:c>
       <x:c r="F181" s="23" t="str">
-        <x:v>Wikipedia (inglés): Harald Bluetooth</x:v>
+        <x:v>Wikipedia (English): Harald Bluetooth</x:v>
       </x:c>
       <x:c r="G181" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Harald_Bluetooth</x:v>
@@ -4485,19 +4485,19 @@
         <x:v>169</x:v>
       </x:c>
       <x:c r="B182" s="23" t="str">
-        <x:v>Jadwiga de Polonia</x:v>
+        <x:v>Jadwiga of Poland</x:v>
       </x:c>
       <x:c r="C182" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D182" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E182" s="23" t="str">
-        <x:v>Polonia</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="F182" s="23" t="str">
-        <x:v>Wikipedia (inglés): Jadwiga of Poland</x:v>
+        <x:v>Wikipedia (English): Jadwiga of Poland</x:v>
       </x:c>
       <x:c r="G182" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Jadwiga_of_Poland</x:v>
@@ -4511,16 +4511,16 @@
         <x:v>Otto von Bismarck</x:v>
       </x:c>
       <x:c r="C183" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D183" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E183" s="23" t="str">
-        <x:v>Prusia / Alemania</x:v>
+        <x:v>Prussia / Germany</x:v>
       </x:c>
       <x:c r="F183" s="23" t="str">
-        <x:v>Wikipedia (inglés): Otto von Bismarck</x:v>
+        <x:v>Wikipedia (English): Otto von Bismarck</x:v>
       </x:c>
       <x:c r="G183" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Otto_von_Bismarck</x:v>
@@ -4531,19 +4531,19 @@
         <x:v>171</x:v>
       </x:c>
       <x:c r="B184" s="23" t="str">
-        <x:v>Juana de Arco</x:v>
+        <x:v>Joan of Arc</x:v>
       </x:c>
       <x:c r="C184" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D184" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E184" s="23" t="str">
-        <x:v>Francia</x:v>
+        <x:v>France</x:v>
       </x:c>
       <x:c r="F184" s="23" t="str">
-        <x:v>Wikipedia (inglés): Joan of Arc</x:v>
+        <x:v>Wikipedia (English): Joan of Arc</x:v>
       </x:c>
       <x:c r="G184" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Joan_of_Arc</x:v>
@@ -4557,16 +4557,16 @@
         <x:v>Giuseppe Garibaldi</x:v>
       </x:c>
       <x:c r="C185" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D185" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E185" s="23" t="str">
-        <x:v>Italia</x:v>
+        <x:v>Italy</x:v>
       </x:c>
       <x:c r="F185" s="23" t="str">
-        <x:v>Wikipedia (inglés): Giuseppe Garibaldi</x:v>
+        <x:v>Wikipedia (English): Giuseppe Garibaldi</x:v>
       </x:c>
       <x:c r="G185" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Giuseppe_Garibaldi</x:v>
@@ -4580,16 +4580,16 @@
         <x:v>Cristina de Suecia</x:v>
       </x:c>
       <x:c r="C186" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D186" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E186" s="23" t="str">
-        <x:v>Suecia</x:v>
+        <x:v>Sweden</x:v>
       </x:c>
       <x:c r="F186" s="23" t="str">
-        <x:v>Wikipedia (inglés): Christina, Queen of Sweden</x:v>
+        <x:v>Wikipedia (English): Christina, Queen of Sweden</x:v>
       </x:c>
       <x:c r="G186" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Christina,_Queen_of_Sweden</x:v>
@@ -4600,19 +4600,19 @@
         <x:v>174</x:v>
       </x:c>
       <x:c r="B187" s="23" t="str">
-        <x:v>Federico el Grande</x:v>
+        <x:v>Frederick the Great</x:v>
       </x:c>
       <x:c r="C187" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D187" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E187" s="23" t="str">
         <x:v>Prusia</x:v>
       </x:c>
       <x:c r="F187" s="23" t="str">
-        <x:v>Wikipedia (inglés): Frederick the Great</x:v>
+        <x:v>Wikipedia (English): Frederick the Great</x:v>
       </x:c>
       <x:c r="G187" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Frederick_the_Great</x:v>
@@ -4623,19 +4623,19 @@
         <x:v>175</x:v>
       </x:c>
       <x:c r="B188" s="23" t="str">
-        <x:v>Catalina de Médici</x:v>
+        <x:v>Catherine de' Medici</x:v>
       </x:c>
       <x:c r="C188" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D188" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E188" s="23" t="str">
-        <x:v>Francia</x:v>
+        <x:v>France</x:v>
       </x:c>
       <x:c r="F188" s="23" t="str">
-        <x:v>Wikipedia (inglés): Catherine de' Medici</x:v>
+        <x:v>Wikipedia (English): Catherine de' Medici</x:v>
       </x:c>
       <x:c r="G188" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Catherine_de%27_Medici</x:v>
@@ -4646,19 +4646,19 @@
         <x:v>176</x:v>
       </x:c>
       <x:c r="B189" s="23" t="str">
-        <x:v>Sviatoslav I de Kiev</x:v>
+        <x:v>Sviatoslav I</x:v>
       </x:c>
       <x:c r="C189" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D189" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E189" s="23" t="str">
-        <x:v>Rus de Kiev</x:v>
+        <x:v>Kievan Rus'</x:v>
       </x:c>
       <x:c r="F189" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sviatoslav I</x:v>
+        <x:v>Wikipedia (English): Sviatoslav I</x:v>
       </x:c>
       <x:c r="G189" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Sviatoslav_I</x:v>
@@ -4669,19 +4669,19 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="B190" s="23" t="str">
-        <x:v>Matilde de Inglaterra</x:v>
+        <x:v>Empress Matilda</x:v>
       </x:c>
       <x:c r="C190" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D190" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E190" s="23" t="str">
-        <x:v>Inglaterra</x:v>
+        <x:v>England</x:v>
       </x:c>
       <x:c r="F190" s="23" t="str">
-        <x:v>Wikipedia (inglés): Empress Matilda</x:v>
+        <x:v>Wikipedia (English): Empress Matilda</x:v>
       </x:c>
       <x:c r="G190" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Empress_Matilda</x:v>
@@ -4695,16 +4695,16 @@
         <x:v>Stefan Dušan</x:v>
       </x:c>
       <x:c r="C191" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D191" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E191" s="23" t="str">
-        <x:v>Imperio serbio</x:v>
+        <x:v>Serbian Empire</x:v>
       </x:c>
       <x:c r="F191" s="23" t="str">
-        <x:v>Wikipedia (inglés): Stefan Dušan</x:v>
+        <x:v>Wikipedia (English): Stefan Dušan</x:v>
       </x:c>
       <x:c r="G191" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Stefan_Du%C5%A1an</x:v>
@@ -4715,19 +4715,19 @@
         <x:v>179</x:v>
       </x:c>
       <x:c r="B192" s="23" t="str">
-        <x:v>Matilde de Toscana</x:v>
+        <x:v>Matilda of Tuscany</x:v>
       </x:c>
       <x:c r="C192" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D192" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E192" s="23" t="str">
-        <x:v>Toscana / Italia</x:v>
+        <x:v>Tuscany / Italy</x:v>
       </x:c>
       <x:c r="F192" s="23" t="str">
-        <x:v>Wikipedia (inglés): Matilda of Tuscany</x:v>
+        <x:v>Wikipedia (English): Matilda of Tuscany</x:v>
       </x:c>
       <x:c r="G192" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Matilda_of_Tuscany</x:v>
@@ -4738,19 +4738,19 @@
         <x:v>180</x:v>
       </x:c>
       <x:c r="B193" s="23" t="str">
-        <x:v>Canuto el Grande</x:v>
+        <x:v>Cnut</x:v>
       </x:c>
       <x:c r="C193" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D193" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E193" s="23" t="str">
-        <x:v>Mar del Norte / Inglaterra y Dinamarca</x:v>
+        <x:v>North Sea / England and Denmark</x:v>
       </x:c>
       <x:c r="F193" s="23" t="str">
-        <x:v>Wikipedia (inglés): Cnut</x:v>
+        <x:v>Wikipedia (English): Cnut</x:v>
       </x:c>
       <x:c r="G193" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Cnut</x:v>
@@ -4761,19 +4761,19 @@
         <x:v>181</x:v>
       </x:c>
       <x:c r="B194" s="23" t="str">
-        <x:v>Fredegunda</x:v>
+        <x:v>Fredegund</x:v>
       </x:c>
       <x:c r="C194" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D194" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E194" s="23" t="str">
-        <x:v>Reino franco</x:v>
+        <x:v>Frankish Kingdom</x:v>
       </x:c>
       <x:c r="F194" s="23" t="str">
-        <x:v>Wikipedia (inglés): Fredegund</x:v>
+        <x:v>Wikipedia (English): Fredegund</x:v>
       </x:c>
       <x:c r="G194" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Fredegund</x:v>
@@ -4787,16 +4787,16 @@
         <x:v>Carlos V</x:v>
       </x:c>
       <x:c r="C195" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D195" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E195" s="23" t="str">
-        <x:v>Sacro Imperio Romano y España</x:v>
+        <x:v>Holy Roman Empire and Spain</x:v>
       </x:c>
       <x:c r="F195" s="23" t="str">
-        <x:v>Wikipedia (inglés): Charles V, Holy Roman Emperor</x:v>
+        <x:v>Wikipedia (English): Charles V, Holy Roman Emperor</x:v>
       </x:c>
       <x:c r="G195" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Charles_V,_Holy_Roman_Emperor</x:v>
@@ -4810,16 +4810,16 @@
         <x:v>Grace O'Malley</x:v>
       </x:c>
       <x:c r="C196" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D196" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E196" s="23" t="str">
-        <x:v>Irlanda</x:v>
+        <x:v>Ireland</x:v>
       </x:c>
       <x:c r="F196" s="23" t="str">
-        <x:v>Wikipedia (inglés): Grace O'Malley</x:v>
+        <x:v>Wikipedia (English): Grace O'Malley</x:v>
       </x:c>
       <x:c r="G196" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Grace_O%27Malley</x:v>
@@ -4830,19 +4830,19 @@
         <x:v>184</x:v>
       </x:c>
       <x:c r="B197" s="23" t="str">
-        <x:v>Esteban el Grande de Moldavia</x:v>
+        <x:v>Stephen the Great</x:v>
       </x:c>
       <x:c r="C197" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D197" s="22" t="str">
-        <x:v>Europa</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E197" s="23" t="str">
         <x:v>Moldavia</x:v>
       </x:c>
       <x:c r="F197" s="23" t="str">
-        <x:v>Wikipedia (inglés): Stephen the Great</x:v>
+        <x:v>Wikipedia (English): Stephen the Great</x:v>
       </x:c>
       <x:c r="G197" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Stephen_the_Great</x:v>
@@ -4856,16 +4856,16 @@
         <x:v>Kaʻahumanu</x:v>
       </x:c>
       <x:c r="C198" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D198" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E198" s="23" t="str">
-        <x:v>Reino de Hawái</x:v>
+        <x:v>Kingdom of Hawaii</x:v>
       </x:c>
       <x:c r="F198" s="23" t="str">
-        <x:v>Wikipedia (inglés): Kaʻahumanu</x:v>
+        <x:v>Wikipedia (English): Kaʻahumanu</x:v>
       </x:c>
       <x:c r="G198" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Ka%CA%BBahumanu</x:v>
@@ -4879,16 +4879,16 @@
         <x:v>Kamehameha I</x:v>
       </x:c>
       <x:c r="C199" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D199" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E199" s="23" t="str">
-        <x:v>Reino de Hawái</x:v>
+        <x:v>Kingdom of Hawaii</x:v>
       </x:c>
       <x:c r="F199" s="23" t="str">
-        <x:v>Wikipedia (inglés): Kamehameha I</x:v>
+        <x:v>Wikipedia (English): Kamehameha I</x:v>
       </x:c>
       <x:c r="G199" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Kamehameha_I</x:v>
@@ -4902,16 +4902,16 @@
         <x:v>Liliʻuokalani</x:v>
       </x:c>
       <x:c r="C200" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D200" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E200" s="23" t="str">
-        <x:v>Reino de Hawái</x:v>
+        <x:v>Kingdom of Hawaii</x:v>
       </x:c>
       <x:c r="F200" s="23" t="str">
-        <x:v>Wikipedia (inglés): Liliʻuokalani</x:v>
+        <x:v>Wikipedia (English): Liliʻuokalani</x:v>
       </x:c>
       <x:c r="G200" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Lili%CA%BBuokalani</x:v>
@@ -4925,16 +4925,16 @@
         <x:v>Hongi Hika</x:v>
       </x:c>
       <x:c r="C201" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D201" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E201" s="23" t="str">
         <x:v>Māori / Ngāpuhi</x:v>
       </x:c>
       <x:c r="F201" s="23" t="str">
-        <x:v>Wikipedia (inglés): Hongi Hika</x:v>
+        <x:v>Wikipedia (English): Hongi Hika</x:v>
       </x:c>
       <x:c r="G201" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Hongi_Hika</x:v>
@@ -4948,16 +4948,16 @@
         <x:v>Pōmare IV</x:v>
       </x:c>
       <x:c r="C202" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D202" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E202" s="23" t="str">
-        <x:v>Tahití</x:v>
+        <x:v>Tahiti</x:v>
       </x:c>
       <x:c r="F202" s="23" t="str">
-        <x:v>Wikipedia (inglés): Pōmare IV</x:v>
+        <x:v>Wikipedia (English): Pōmare IV</x:v>
       </x:c>
       <x:c r="G202" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/P%C5%8Dmare_IV</x:v>
@@ -4971,16 +4971,16 @@
         <x:v>Te Rauparaha</x:v>
       </x:c>
       <x:c r="C203" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D203" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E203" s="23" t="str">
         <x:v>Māori / Ngāti Toa</x:v>
       </x:c>
       <x:c r="F203" s="23" t="str">
-        <x:v>Wikipedia (inglés): Te Rauparaha</x:v>
+        <x:v>Wikipedia (English): Te Rauparaha</x:v>
       </x:c>
       <x:c r="G203" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Te_Rauparaha</x:v>
@@ -4994,16 +4994,16 @@
         <x:v>Sālote Tupou III</x:v>
       </x:c>
       <x:c r="C204" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D204" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E204" s="23" t="str">
         <x:v>Tonga</x:v>
       </x:c>
       <x:c r="F204" s="23" t="str">
-        <x:v>Wikipedia (inglés): Sālote Tupou III</x:v>
+        <x:v>Wikipedia (English): Sālote Tupou III</x:v>
       </x:c>
       <x:c r="G204" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/S%C4%81lote_Tupou_III</x:v>
@@ -5017,16 +5017,16 @@
         <x:v>Pōtatau Te Wherowhero</x:v>
       </x:c>
       <x:c r="C205" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D205" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E205" s="23" t="str">
         <x:v>Māori / Waikato</x:v>
       </x:c>
       <x:c r="F205" s="23" t="str">
-        <x:v>Wikipedia (inglés): Pōtatau Te Wherowhero</x:v>
+        <x:v>Wikipedia (English): Pōtatau Te Wherowhero</x:v>
       </x:c>
       <x:c r="G205" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/P%C5%8Dtatau_Te_Wherowhero</x:v>
@@ -5040,16 +5040,16 @@
         <x:v>Te Puea Hērangi</x:v>
       </x:c>
       <x:c r="C206" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D206" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E206" s="23" t="str">
         <x:v>Māori / Waikato</x:v>
       </x:c>
       <x:c r="F206" s="23" t="str">
-        <x:v>Wikipedia (inglés): Te Puea Hērangi</x:v>
+        <x:v>Wikipedia (English): Te Puea Hērangi</x:v>
       </x:c>
       <x:c r="G206" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Te_Puea_H%C4%93rangi</x:v>
@@ -5063,16 +5063,16 @@
         <x:v>Tāmati Wāka Nene</x:v>
       </x:c>
       <x:c r="C207" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D207" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E207" s="23" t="str">
         <x:v>Māori / Ngāpuhi</x:v>
       </x:c>
       <x:c r="F207" s="23" t="str">
-        <x:v>Wikipedia (inglés): Tāmati Wāka Nene</x:v>
+        <x:v>Wikipedia (English): Tāmati Wāka Nene</x:v>
       </x:c>
       <x:c r="G207" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/T%C4%81mati_W%C4%81ka_Nene</x:v>
@@ -5086,16 +5086,16 @@
         <x:v>Whina Cooper</x:v>
       </x:c>
       <x:c r="C208" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D208" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E208" s="23" t="str">
         <x:v>Māori / Aotearoa</x:v>
       </x:c>
       <x:c r="F208" s="23" t="str">
-        <x:v>Wikipedia (inglés): Whina Cooper</x:v>
+        <x:v>Wikipedia (English): Whina Cooper</x:v>
       </x:c>
       <x:c r="G208" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Whina_Cooper</x:v>
@@ -5109,16 +5109,16 @@
         <x:v>Pemulwuy</x:v>
       </x:c>
       <x:c r="C209" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D209" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E209" s="23" t="str">
-        <x:v>Pueblo bidjigal / Australia</x:v>
+        <x:v>Bidjigal people / Australia</x:v>
       </x:c>
       <x:c r="F209" s="23" t="str">
-        <x:v>Wikipedia (inglés): Pemulwuy</x:v>
+        <x:v>Wikipedia (English): Pemulwuy</x:v>
       </x:c>
       <x:c r="G209" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Pemulwuy</x:v>
@@ -5132,16 +5132,16 @@
         <x:v>Makea Takau Ariki</x:v>
       </x:c>
       <x:c r="C210" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D210" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E210" s="23" t="str">
-        <x:v>Rarotonga / Islas Cook</x:v>
+        <x:v>Rarotonga / Cook Islands</x:v>
       </x:c>
       <x:c r="F210" s="23" t="str">
-        <x:v>Wikipedia (inglés): Makea Takau Ariki</x:v>
+        <x:v>Wikipedia (English): Makea Takau Ariki</x:v>
       </x:c>
       <x:c r="G210" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Makea_Takau_Ariki</x:v>
@@ -5155,16 +5155,16 @@
         <x:v>Yagan</x:v>
       </x:c>
       <x:c r="C211" s="22" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D211" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E211" s="23" t="str">
-        <x:v>Pueblo noongar / Australia</x:v>
+        <x:v>Noongar people / Australia</x:v>
       </x:c>
       <x:c r="F211" s="23" t="str">
-        <x:v>Wikipedia (inglés): Yagan</x:v>
+        <x:v>Wikipedia (English): Yagan</x:v>
       </x:c>
       <x:c r="G211" s="24" t="str">
         <x:v>https://en.wikipedia.org/wiki/Yagan</x:v>
@@ -5178,10 +5178,10 @@
         <x:v>Maria Angata</x:v>
       </x:c>
       <x:c r="C212" s="22" t="str">
-        <x:v>Mujer</x:v>
+        <x:v>Woman</x:v>
       </x:c>
       <x:c r="D212" s="22" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E212" s="23" t="str">
         <x:v>Rapa Nui</x:v>
@@ -5201,16 +5201,16 @@
         <x:v>George Tupou I</x:v>
       </x:c>
       <x:c r="C213" s="25" t="str">
-        <x:v>Hombre</x:v>
+        <x:v>Man</x:v>
       </x:c>
       <x:c r="D213" s="25" t="str">
-        <x:v>Oceanía</x:v>
+        <x:v>Oceania</x:v>
       </x:c>
       <x:c r="E213" s="26" t="str">
         <x:v>Tonga</x:v>
       </x:c>
       <x:c r="F213" s="26" t="str">
-        <x:v>Wikipedia (inglés): George Tupou I</x:v>
+        <x:v>Wikipedia (English): George Tupou I</x:v>
       </x:c>
       <x:c r="G213" s="27" t="str">
         <x:v>https://en.wikipedia.org/wiki/George_Tupou_I</x:v>

</xml_diff>